<commit_message>
Update PO static site data
</commit_message>
<xml_diff>
--- a/output/public_agency_subsidiaries.xlsx
+++ b/output/public_agency_subsidiaries.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A694"/>
+  <dimension ref="A1:A646"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1063,4212 +1063,3876 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>BANCOKDBDOBRASILS.A.</t>
+          <t>BusanPortAuthorityB.V.</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>BusanPortAuthorityB.V.</t>
+          <t>ChitoseSolarPowerPlantLLC</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>ChitoseSolarPowerPlantLLC</t>
+          <t>DanaPetroleumLtd.</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>DKIGrowingStar3호투자조합</t>
+          <t>EWP(Barbados)1SRL</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>DSC유망서비스산업펀드</t>
+          <t>EWPAmerica, Inc.</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>DanaPetroleumLtd.</t>
+          <t>EWPAustraliaPtyLtd</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>EWP(Barbados)1SRL</t>
+          <t>EWPBylongPtyLimited</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>EWPAmerica, Inc.</t>
+          <t>ErmaniLtd.</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>EWPAustraliaPtyLtd</t>
+          <t>FujeijWindPowerCompany</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>EWPBylongPtyLimited</t>
+          <t>GLOBALKOMSCODAEWOOLLC.</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>ErmaniLtd.</t>
+          <t>GlobalEnergyPioneerB.V.</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>FujeijWindPowerCompany</t>
+          <t>GlobalOnePioneerB.V.</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>GLOBALKOMSCODAEWOOLLC.</t>
+          <t>GuamUkuduPowerLLC</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>GlobalEnergyPioneerB.V.</t>
+          <t>HarvestOperationsCorp</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>GlobalOnePioneerB.V.</t>
+          <t>IBK-스톤브릿지라이징2호투자조합</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>GuamUkuduPowerLLC</t>
+          <t>IBK금융그룹미래성장동력투자조합</t>
         </is>
       </c>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>HarvestOperationsCorp</t>
+          <t>IBK금융그룹창업기업일자리창출투자조합</t>
         </is>
       </c>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>IBK-스톤브릿지라이징2호투자조합</t>
+          <t>IBK금융그룹크라우드펀딩매칭투자조합</t>
         </is>
       </c>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>IBK금융그룹미래성장동력투자조합</t>
+          <t>IBK미얀마은행</t>
         </is>
       </c>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>IBK금융그룹창업기업일자리창출투자조합</t>
+          <t>IBK신용정보㈜</t>
         </is>
       </c>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>IBK금융그룹크라우드펀딩매칭투자조합</t>
+          <t>IBK연금보험㈜</t>
         </is>
       </c>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>IBK미얀마은행</t>
+          <t>IBK인도네시아은행</t>
         </is>
       </c>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>IBK신용정보㈜</t>
+          <t>IBK자산운용㈜</t>
         </is>
       </c>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>IBK연금보험㈜</t>
+          <t>IBK창공비상1호투자조합</t>
         </is>
       </c>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>IBK인도네시아은행</t>
+          <t>IBK창공비상2호투자조합</t>
         </is>
       </c>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>IBK자산운용㈜</t>
+          <t>IBK투자증권㈜</t>
         </is>
       </c>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>IBK창공비상1호투자조합</t>
+          <t>IBK폴란드은행</t>
         </is>
       </c>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>IBK창공비상2호투자조합</t>
+          <t>IPKoreaCenterInc</t>
         </is>
       </c>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>IBK투자증권㈜</t>
+          <t>IncheonAirportPhilippinesCorporation</t>
         </is>
       </c>
     </row>
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>IBK폴란드은행</t>
+          <t>IncheonKoreaforAirportServicesCompanyS.P.C</t>
         </is>
       </c>
     </row>
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>IPKoreaCenterInc</t>
+          <t>JSCNenskraHydro</t>
         </is>
       </c>
     </row>
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>IncheonAirportPhilippinesCorporation</t>
+          <t>KADOCLtd.</t>
         </is>
       </c>
     </row>
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>IncheonKoreaforAirportServicesCompanyS.P.C</t>
+          <t>KAPowerLimited</t>
         </is>
       </c>
     </row>
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>JSCKDBBANKUZBEKISTAN</t>
+          <t>KDSHydroPte. Ltd.</t>
         </is>
       </c>
     </row>
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>JSCNenskraHydro</t>
+          <t>KEPCOAustraliaPty., Ltd.</t>
         </is>
       </c>
     </row>
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>KADOCLtd.</t>
+          <t>KEPCOCalifornia, LLC</t>
         </is>
       </c>
     </row>
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>KAPowerLimited</t>
+          <t>KEPCOGansuInternationalLtd.</t>
         </is>
       </c>
     </row>
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>KDBASIALIMITED</t>
+          <t>KEPCOHoldingCompany</t>
         </is>
       </c>
     </row>
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>KDBBANKEUROPELIMITED</t>
+          <t>KEPCOHoldingsdeMexico</t>
         </is>
       </c>
     </row>
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>KDBC공동투자사모투자합자회사</t>
+          <t>KEPCOInternationalHongKongLtd.</t>
         </is>
       </c>
     </row>
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>KDBIRELANDDESIGNATEDACTIVITYCOMPANY</t>
+          <t>KEPCOInternationalPhilippinesInc.</t>
         </is>
       </c>
     </row>
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>KDBOCCASIOII, L.P.</t>
+          <t>KEPCOKPSPhilippinesCorp.</t>
         </is>
       </c>
     </row>
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>KDBSILICONVALLEYLLC</t>
+          <t>KEPCOKPSSouthAfricaPty., Ltd.</t>
         </is>
       </c>
     </row>
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>KDBSynergy, L.P.</t>
+          <t>KEPCOMangilaoHoldingsLLC</t>
         </is>
       </c>
     </row>
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>KDSHydroPte. Ltd.</t>
+          <t>KEPCOMiddleEastHoldingCompany</t>
         </is>
       </c>
     </row>
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>KEPCOAustraliaPty., Ltd.</t>
+          <t>KEPCONeimengguInternationalLtd.</t>
         </is>
       </c>
     </row>
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>KEPCOCalifornia, LLC</t>
+          <t>KEPCONetherlandsB.V.</t>
         </is>
       </c>
     </row>
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t>KEPCOGansuInternationalLtd.</t>
+          <t>KEPCONetherlandsJ3B.V.</t>
         </is>
       </c>
     </row>
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t>KEPCOHoldingCompany</t>
+          <t>KEPCONetherlandsS3B.V.</t>
         </is>
       </c>
     </row>
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>KEPCOHoldingsdeMexico</t>
+          <t>KEPCOPhilippinesHoldingsInc.</t>
         </is>
       </c>
     </row>
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>KEPCOInternationalHongKongLtd.</t>
+          <t>KEPCOSADAWI - FZCO</t>
         </is>
       </c>
     </row>
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>KEPCOInternationalPhilippinesInc.</t>
+          <t>KEPCOShanxiInternationalLtd.</t>
         </is>
       </c>
     </row>
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>KEPCOKPSPhilippinesCorp.</t>
+          <t>KEPCOYonaAmericaLLC</t>
         </is>
       </c>
     </row>
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>KEPCOKPSSouthAfricaPty., Ltd.</t>
+          <t>KG-SEAGPCompanyLimited</t>
         </is>
       </c>
     </row>
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>KEPCOMangilaoHoldingsLLC</t>
+          <t>KGKruengManeLtd.</t>
         </is>
       </c>
     </row>
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>KEPCOMiddleEastHoldingCompany</t>
+          <t>KGMozambiqueLtd.</t>
         </is>
       </c>
     </row>
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>KEPCONeimengguInternationalLtd.</t>
+          <t>KHNPCanadaEnergyLtd.</t>
         </is>
       </c>
     </row>
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>KEPCONetherlandsB.V.</t>
+          <t>KHNPChileSpA</t>
         </is>
       </c>
     </row>
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t>KEPCONetherlandsJ3B.V.</t>
+          <t>KHNPUSALLC</t>
         </is>
       </c>
     </row>
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>KEPCONetherlandsS3B.V.</t>
+          <t>KINDUSALLC</t>
         </is>
       </c>
     </row>
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>KEPCOPhilippinesHoldingsInc.</t>
+          <t>KNFCanadaEnergyLtd.</t>
         </is>
       </c>
     </row>
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
-          <t>KEPCOSADAWI - FZCO</t>
+          <t>KNOCEaglefordCorp.</t>
         </is>
       </c>
     </row>
     <row r="155">
       <c r="A155" t="inlineStr">
         <is>
-          <t>KEPCOShanxiInternationalLtd.</t>
+          <t>KNOCKazB.V.</t>
         </is>
       </c>
     </row>
     <row r="156">
       <c r="A156" t="inlineStr">
         <is>
-          <t>KEPCOYonaAmericaLLC</t>
+          <t>KNOCNigerianEastOilCompanyLtd.</t>
         </is>
       </c>
     </row>
     <row r="157">
       <c r="A157" t="inlineStr">
         <is>
-          <t>KG-SEAGPCompanyLimited</t>
+          <t>KNOCNigerianWestOilCompanyLtd.</t>
         </is>
       </c>
     </row>
     <row r="158">
       <c r="A158" t="inlineStr">
         <is>
-          <t>KGKruengManeLtd.</t>
+          <t>KNOCSumatraLtd.</t>
         </is>
       </c>
     </row>
     <row r="159">
       <c r="A159" t="inlineStr">
         <is>
-          <t>KGMozambiqueLtd.</t>
+          <t>KNOCTradingSingapore.Pte.Ltd</t>
         </is>
       </c>
     </row>
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t>KHNPCanadaEnergyLtd.</t>
+          <t>KNOCYemenLtd.</t>
         </is>
       </c>
     </row>
     <row r="161">
       <c r="A161" t="inlineStr">
         <is>
-          <t>KHNPChileSpA</t>
+          <t>KOAKPowerLimited</t>
         </is>
       </c>
     </row>
     <row r="162">
       <c r="A162" t="inlineStr">
         <is>
-          <t>KHNPUSALLC</t>
+          <t>KOBCCONTAINERLEASINGNO. 1LIMITED</t>
         </is>
       </c>
     </row>
     <row r="163">
       <c r="A163" t="inlineStr">
         <is>
-          <t>KINDUSALLC</t>
+          <t>KOBCCONTAINERLEASINGNO. 2LIMITED</t>
         </is>
       </c>
     </row>
     <row r="164">
       <c r="A164" t="inlineStr">
         <is>
-          <t>KNFCanadaEnergyLtd.</t>
+          <t>KOBCCONTAINERLEASINGNO. 3LIMITED</t>
         </is>
       </c>
     </row>
     <row r="165">
       <c r="A165" t="inlineStr">
         <is>
-          <t>KNOCEaglefordCorp.</t>
+          <t>KOBCUSALLC</t>
         </is>
       </c>
     </row>
     <row r="166">
       <c r="A166" t="inlineStr">
         <is>
-          <t>KNOCKazB.V.</t>
+          <t>KOENBylongPty., Ltd.</t>
         </is>
       </c>
     </row>
     <row r="167">
       <c r="A167" t="inlineStr">
         <is>
-          <t>KNOCNigerianEastOilCompanyLtd.</t>
+          <t>KOFPI.PARAGUAY.S.A</t>
         </is>
       </c>
     </row>
     <row r="168">
       <c r="A168" t="inlineStr">
         <is>
-          <t>KNOCNigerianWestOilCompanyLtd.</t>
+          <t>KOGAMEXInvestmentManzanilloB.V.</t>
         </is>
       </c>
     </row>
     <row r="169">
       <c r="A169" t="inlineStr">
         <is>
-          <t>KNOCSumatraLtd.</t>
+          <t>KOGASAkkasB.V.</t>
         </is>
       </c>
     </row>
     <row r="170">
       <c r="A170" t="inlineStr">
         <is>
-          <t>KNOCTradingSingapore.Pte.Ltd</t>
+          <t>KOGASAustraliaPty. Ltd.</t>
         </is>
       </c>
     </row>
     <row r="171">
       <c r="A171" t="inlineStr">
         <is>
-          <t>KNOCYemenLtd.</t>
+          <t>KOGASBadraB.V.</t>
         </is>
       </c>
     </row>
     <row r="172">
       <c r="A172" t="inlineStr">
         <is>
-          <t>KOAKPowerLimited</t>
+          <t>KOGASCanadaEnergyLtd.</t>
         </is>
       </c>
     </row>
     <row r="173">
       <c r="A173" t="inlineStr">
         <is>
-          <t>KOBCCONTAINERLEASINGNO. 1LIMITED</t>
+          <t>KOGASCyprusLtd.</t>
         </is>
       </c>
     </row>
     <row r="174">
       <c r="A174" t="inlineStr">
         <is>
-          <t>KOBCCONTAINERLEASINGNO. 2LIMITED</t>
+          <t>KOGASInternationalPte. Ltd.</t>
         </is>
       </c>
     </row>
     <row r="175">
       <c r="A175" t="inlineStr">
         <is>
-          <t>KOBCCONTAINERLEASINGNO. 3LIMITED</t>
+          <t>KOGASIraqB.V.</t>
         </is>
       </c>
     </row>
     <row r="176">
       <c r="A176" t="inlineStr">
         <is>
-          <t>KOBCUSALLC</t>
+          <t>KOGASMansuriyaB.V.</t>
         </is>
       </c>
     </row>
     <row r="177">
       <c r="A177" t="inlineStr">
         <is>
-          <t>KOENBylongPty., Ltd.</t>
+          <t>KOGASMozambiqueLda.</t>
         </is>
       </c>
     </row>
     <row r="178">
       <c r="A178" t="inlineStr">
         <is>
-          <t>KOFPI.PARAGUAY.S.A</t>
+          <t>KOGASPreludePty. Ltd.</t>
         </is>
       </c>
     </row>
     <row r="179">
       <c r="A179" t="inlineStr">
         <is>
-          <t>KOGAMEXInvestmentManzanilloB.V.</t>
+          <t>KOLATSpA</t>
         </is>
       </c>
     </row>
     <row r="180">
       <c r="A180" t="inlineStr">
         <is>
-          <t>KOGASAkkasB.V.</t>
+          <t>KOMEX-GAS, S. deR. L. deC.V.(주3)</t>
         </is>
       </c>
     </row>
     <row r="181">
       <c r="A181" t="inlineStr">
         <is>
-          <t>KOGASAustraliaPty. Ltd.</t>
+          <t>KOMIPOAmericaInc.</t>
         </is>
       </c>
     </row>
     <row r="182">
       <c r="A182" t="inlineStr">
         <is>
-          <t>KOGASBadraB.V.</t>
+          <t>KOMIPOAustraliaPtyLtd.</t>
         </is>
       </c>
     </row>
     <row r="183">
       <c r="A183" t="inlineStr">
         <is>
-          <t>KOGASCanadaEnergyLtd.</t>
+          <t>KOMIPOBylongPtyLtd</t>
         </is>
       </c>
     </row>
     <row r="184">
       <c r="A184" t="inlineStr">
         <is>
-          <t>KOGASCyprusLtd.</t>
+          <t>KOMIPOEuropeB.V.</t>
         </is>
       </c>
     </row>
     <row r="185">
       <c r="A185" t="inlineStr">
         <is>
-          <t>KOGASInternationalPte. Ltd.</t>
+          <t>KOMIPOGlobalPteLtd.</t>
         </is>
       </c>
     </row>
     <row r="186">
       <c r="A186" t="inlineStr">
         <is>
-          <t>KOGASIraqB.V.</t>
+          <t>KOMIPOVanPhongPowerServiceLLC</t>
         </is>
       </c>
     </row>
     <row r="187">
       <c r="A187" t="inlineStr">
         <is>
-          <t>KOGASMansuriyaB.V.</t>
+          <t>KORESCANADACorp.</t>
         </is>
       </c>
     </row>
     <row r="188">
       <c r="A188" t="inlineStr">
         <is>
-          <t>KOGASMozambiqueLda.</t>
+          <t>KOSEPAustraliaPty.,Ltd.</t>
         </is>
       </c>
     </row>
     <row r="189">
       <c r="A189" t="inlineStr">
         <is>
-          <t>KOGASPreludePty. Ltd.</t>
+          <t>KOSPOAustraliaPty., Ltd.</t>
         </is>
       </c>
     </row>
     <row r="190">
       <c r="A190" t="inlineStr">
         <is>
-          <t>KOLATSpA</t>
+          <t>KOSPOBylongPty., Ltd.</t>
         </is>
       </c>
     </row>
     <row r="191">
       <c r="A191" t="inlineStr">
         <is>
-          <t>KOMEX-GAS, S. deR. L. deC.V.(주3)</t>
+          <t>KOSPOChileSpA</t>
         </is>
       </c>
     </row>
     <row r="192">
       <c r="A192" t="inlineStr">
         <is>
-          <t>KOMIPOAmericaInc.</t>
+          <t>KOSPOJORDANL.L.C.</t>
         </is>
       </c>
     </row>
     <row r="193">
       <c r="A193" t="inlineStr">
         <is>
-          <t>KOMIPOAustraliaPtyLtd.</t>
+          <t>KOSPOUSAInc.</t>
         </is>
       </c>
     </row>
     <row r="194">
       <c r="A194" t="inlineStr">
         <is>
-          <t>KOMIPOBylongPtyLtd</t>
+          <t>KOWEPOAustraliaPty.,Ltd.</t>
         </is>
       </c>
     </row>
     <row r="195">
       <c r="A195" t="inlineStr">
         <is>
-          <t>KOMIPOEuropeB.V.</t>
+          <t>KOWEPOBylongPty.,Ltd</t>
         </is>
       </c>
     </row>
     <row r="196">
       <c r="A196" t="inlineStr">
         <is>
-          <t>KOMIPOGlobalPteLtd.</t>
+          <t>KOWEPOEuropeB.V.</t>
         </is>
       </c>
     </row>
     <row r="197">
       <c r="A197" t="inlineStr">
         <is>
-          <t>KOMIPOVanPhongPowerServiceLLC</t>
+          <t>KOWEPOHoldingLimited</t>
         </is>
       </c>
     </row>
     <row r="198">
       <c r="A198" t="inlineStr">
         <is>
-          <t>KORESCANADACorp.</t>
+          <t>KOWEPOInternationalCorporation</t>
         </is>
       </c>
     </row>
     <row r="199">
       <c r="A199" t="inlineStr">
         <is>
-          <t>KOSEPAustraliaPty.,Ltd.</t>
+          <t>KOWEPOLaoInternational</t>
         </is>
       </c>
     </row>
     <row r="200">
       <c r="A200" t="inlineStr">
         <is>
-          <t>KOSPOAustraliaPty., Ltd.</t>
+          <t>KRCThailand. Co.Ltd</t>
         </is>
       </c>
     </row>
     <row r="201">
       <c r="A201" t="inlineStr">
         <is>
-          <t>KOSPOBylongPty., Ltd.</t>
+          <t>KSTElectricPowerCompany, S.A.P.I. deC.V.</t>
         </is>
       </c>
     </row>
     <row r="202">
       <c r="A202" t="inlineStr">
         <is>
-          <t>KOSPOChileSpA</t>
+          <t>KTLChinaCo.,Ltd</t>
         </is>
       </c>
     </row>
     <row r="203">
       <c r="A203" t="inlineStr">
         <is>
-          <t>KOSPOJORDANL.L.C.</t>
+          <t>KVICASIAPTELTD</t>
         </is>
       </c>
     </row>
     <row r="204">
       <c r="A204" t="inlineStr">
         <is>
-          <t>KOSPOUSAInc.</t>
+          <t>KVICSILICONVALLEYInc</t>
         </is>
       </c>
     </row>
     <row r="205">
       <c r="A205" t="inlineStr">
         <is>
-          <t>KOWEPOAustraliaPty.,Ltd.</t>
+          <t>KoreaRasLaffanLNGLtd.(주1)</t>
         </is>
       </c>
     </row>
     <row r="206">
       <c r="A206" t="inlineStr">
         <is>
-          <t>KOWEPOBylongPty.,Ltd</t>
+          <t>KoreanBoleoCorp</t>
         </is>
       </c>
     </row>
     <row r="207">
       <c r="A207" t="inlineStr">
         <is>
-          <t>KOWEPOEuropeB.V.</t>
+          <t>KoresAustraliaPtyLtd</t>
         </is>
       </c>
     </row>
     <row r="208">
       <c r="A208" t="inlineStr">
         <is>
-          <t>KOWEPOHoldingLimited</t>
+          <t>LHPRIMORYE, LLC</t>
         </is>
       </c>
     </row>
     <row r="209">
       <c r="A209" t="inlineStr">
         <is>
-          <t>KOWEPOInternationalCorporation</t>
+          <t>LSGHydroPowerLtd.</t>
         </is>
       </c>
     </row>
     <row r="210">
       <c r="A210" t="inlineStr">
         <is>
-          <t>KOWEPOLaoInternational</t>
+          <t>MiraPowerLimited</t>
         </is>
       </c>
     </row>
     <row r="211">
       <c r="A211" t="inlineStr">
         <is>
-          <t>KRCThailand. Co.Ltd</t>
+          <t>NepalWater&amp;EnergyDevelopmentCompanyPty.,Ltd.</t>
         </is>
       </c>
     </row>
     <row r="212">
       <c r="A212" t="inlineStr">
         <is>
-          <t>KSTElectricPowerCompany, S.A.P.I. deC.V.</t>
+          <t>PT. EWPIndonesia</t>
         </is>
       </c>
     </row>
     <row r="213">
       <c r="A213" t="inlineStr">
         <is>
-          <t>KTLChinaCo.,Ltd</t>
+          <t>PT. KOMIPOEnergyIndonesia</t>
         </is>
       </c>
     </row>
     <row r="214">
       <c r="A214" t="inlineStr">
         <is>
-          <t>KVICASIAPTELTD</t>
+          <t>PT. KOMIPOPembangkitanJawaBali</t>
         </is>
       </c>
     </row>
     <row r="215">
       <c r="A215" t="inlineStr">
         <is>
-          <t>KVICSILICONVALLEYInc</t>
+          <t>PT. MitraIncheonIndonesia</t>
         </is>
       </c>
     </row>
     <row r="216">
       <c r="A216" t="inlineStr">
         <is>
-          <t>KoFC-BKPioneerChamp2010-13호투자조합</t>
+          <t>PT. koreaEnergyIndonesia</t>
         </is>
       </c>
     </row>
     <row r="217">
       <c r="A217" t="inlineStr">
         <is>
-          <t>KoFC-KVIC일자리창출펀드2호</t>
+          <t>PTHasangOperationandMaintenance</t>
         </is>
       </c>
     </row>
     <row r="218">
       <c r="A218" t="inlineStr">
         <is>
-          <t>KoreaRasLaffanLNGLtd.(주1)</t>
+          <t>PTKarianWaterServices</t>
         </is>
       </c>
     </row>
     <row r="219">
       <c r="A219" t="inlineStr">
         <is>
-          <t>KoreanBoleoCorp</t>
+          <t>PatrindO&amp;M(Private)Limited</t>
         </is>
       </c>
     </row>
     <row r="220">
       <c r="A220" t="inlineStr">
         <is>
-          <t>KoresAustraliaPtyLtd</t>
+          <t>RESTechnologyAD</t>
         </is>
       </c>
     </row>
     <row r="221">
       <c r="A221" t="inlineStr">
         <is>
-          <t>LHPRIMORYE, LLC</t>
+          <t>TinaHydropowerLimited</t>
         </is>
       </c>
     </row>
     <row r="222">
       <c r="A222" t="inlineStr">
         <is>
-          <t>LSGHydroPowerLtd.</t>
+          <t>㈜ 경기리츠공공임대제1호위탁관리부동산투자회사</t>
         </is>
       </c>
     </row>
     <row r="223">
       <c r="A223" t="inlineStr">
         <is>
-          <t>MiraPowerLimited</t>
+          <t>㈜ 엔에이치에프제16호공공임대위탁관리부동산투자회사</t>
         </is>
       </c>
     </row>
     <row r="224">
       <c r="A224" t="inlineStr">
         <is>
-          <t>NepalWater&amp;EnergyDevelopmentCompanyPty.,Ltd.</t>
+          <t>㈜ 코엔서비스</t>
         </is>
       </c>
     </row>
     <row r="225">
       <c r="A225" t="inlineStr">
         <is>
-          <t>PT. EWPIndonesia</t>
+          <t>㈜IBK벤처투자</t>
         </is>
       </c>
     </row>
     <row r="226">
       <c r="A226" t="inlineStr">
         <is>
-          <t>PT. KOMIPOEnergyIndonesia</t>
+          <t>㈜IBK서비스</t>
         </is>
       </c>
     </row>
     <row r="227">
       <c r="A227" t="inlineStr">
         <is>
-          <t>PT. KOMIPOPembangkitanJawaBali</t>
+          <t>㈜IBK시스템</t>
         </is>
       </c>
     </row>
     <row r="228">
       <c r="A228" t="inlineStr">
         <is>
-          <t>PT. MitraIncheonIndonesia</t>
+          <t>㈜IBK저축은행</t>
         </is>
       </c>
     </row>
     <row r="229">
       <c r="A229" t="inlineStr">
         <is>
-          <t>PT. koreaEnergyIndonesia</t>
+          <t>㈜IBK캐피탈</t>
         </is>
       </c>
     </row>
     <row r="230">
       <c r="A230" t="inlineStr">
         <is>
-          <t>PTHasangOperationandMaintenance</t>
+          <t>㈜국민행복주택제1호위탁관리부동산투자회사</t>
         </is>
       </c>
     </row>
     <row r="231">
       <c r="A231" t="inlineStr">
         <is>
-          <t>PTKDBTIFAFINANCETBK</t>
+          <t>㈜국민행복주택제2호위탁관리부동산투자회사</t>
         </is>
       </c>
     </row>
     <row r="232">
       <c r="A232" t="inlineStr">
         <is>
-          <t>PTKarianWaterServices</t>
+          <t>㈜뉴스테이허브제1호위탁관리부동산투자회사</t>
         </is>
       </c>
     </row>
     <row r="233">
       <c r="A233" t="inlineStr">
         <is>
-          <t>PatrindO&amp;M(Private)Limited</t>
+          <t>㈜뉴스테이허브제2호위탁관리부동산투자회사</t>
         </is>
       </c>
     </row>
     <row r="234">
       <c r="A234" t="inlineStr">
         <is>
-          <t>RESTechnologyAD</t>
+          <t>㈜뉴스테이허브제3호위탁관리부동산투자회사</t>
         </is>
       </c>
     </row>
     <row r="235">
       <c r="A235" t="inlineStr">
         <is>
-          <t>SLI소재부품투자펀드2014-1호</t>
+          <t>㈜대한제1호뉴스테이위탁관리부동산투자회사</t>
         </is>
       </c>
     </row>
     <row r="236">
       <c r="A236" t="inlineStr">
         <is>
-          <t>TinaHydropowerLimited</t>
+          <t>㈜동탄2대우코크렙뉴스테이기업형임대위탁관리부동산투자회사</t>
         </is>
       </c>
     </row>
     <row r="237">
       <c r="A237" t="inlineStr">
         <is>
-          <t>㈜ 경기리츠공공임대제1호위탁관리부동산투자회사</t>
+          <t>㈜민간임대허브제4호위탁관리부동산투자회사</t>
         </is>
       </c>
     </row>
     <row r="238">
       <c r="A238" t="inlineStr">
         <is>
-          <t>㈜ 엔에이치에프제16호공공임대위탁관리부동산투자회사</t>
+          <t>㈜민간임대허브제5호위탁관리부동산투자회사</t>
         </is>
       </c>
     </row>
     <row r="239">
       <c r="A239" t="inlineStr">
         <is>
-          <t>㈜ 코엔서비스</t>
+          <t>㈜민간임대허브제6호위탁관리부동산투자회사</t>
         </is>
       </c>
     </row>
     <row r="240">
       <c r="A240" t="inlineStr">
         <is>
-          <t>㈜IBK벤처투자</t>
+          <t>㈜민간임대허브제7호위탁관리부동산투자회사</t>
         </is>
       </c>
     </row>
     <row r="241">
       <c r="A241" t="inlineStr">
         <is>
-          <t>㈜IBK서비스</t>
+          <t>㈜민간임대허브제8호위탁관리부동산투자회사</t>
         </is>
       </c>
     </row>
     <row r="242">
       <c r="A242" t="inlineStr">
         <is>
-          <t>㈜IBK시스템</t>
+          <t>㈜서울리츠임대주택제1호위탁관리부동산투자회사</t>
         </is>
       </c>
     </row>
     <row r="243">
       <c r="A243" t="inlineStr">
         <is>
-          <t>㈜IBK저축은행</t>
+          <t>㈜서울사회주택토지지원위탁관리부동산투자회사</t>
         </is>
       </c>
     </row>
     <row r="244">
       <c r="A244" t="inlineStr">
         <is>
-          <t>㈜IBK캐피탈</t>
+          <t>㈜에스이그린에너지</t>
         </is>
       </c>
     </row>
     <row r="245">
       <c r="A245" t="inlineStr">
         <is>
-          <t>㈜국민행복주택제1호위탁관리부동산투자회사</t>
+          <t>㈜에이치엘제2호위탁관리부동산투자회사</t>
         </is>
       </c>
     </row>
     <row r="246">
       <c r="A246" t="inlineStr">
         <is>
-          <t>㈜국민행복주택제2호위탁관리부동산투자회사</t>
+          <t>㈜에이치엘제5호위탁관리부동산투자회사</t>
         </is>
       </c>
     </row>
     <row r="247">
       <c r="A247" t="inlineStr">
         <is>
-          <t>㈜뉴스테이허브제1호위탁관리부동산투자회사</t>
+          <t>㈜에이팸</t>
         </is>
       </c>
     </row>
     <row r="248">
       <c r="A248" t="inlineStr">
         <is>
-          <t>㈜뉴스테이허브제2호위탁관리부동산투자회사</t>
+          <t>㈜엔에이치에프제10호공공임대위탁관리부동산투자회사</t>
         </is>
       </c>
     </row>
     <row r="249">
       <c r="A249" t="inlineStr">
         <is>
-          <t>㈜뉴스테이허브제3호위탁관리부동산투자회사</t>
+          <t>㈜엔에이치에프제11호공공임대위탁관리부동산투자회사</t>
         </is>
       </c>
     </row>
     <row r="250">
       <c r="A250" t="inlineStr">
         <is>
-          <t>㈜대한제1호뉴스테이위탁관리부동산투자회사</t>
+          <t>㈜엔에이치에프제12호공공임대위탁관리부동산투자회사</t>
         </is>
       </c>
     </row>
     <row r="251">
       <c r="A251" t="inlineStr">
         <is>
-          <t>㈜동탄2대우코크렙뉴스테이기업형임대위탁관리부동산투자회사</t>
+          <t>㈜엔에이치에프제13호공공임대위탁관리부동산투자회사</t>
         </is>
       </c>
     </row>
     <row r="252">
       <c r="A252" t="inlineStr">
         <is>
-          <t>㈜민간임대허브제4호위탁관리부동산투자회사</t>
+          <t>㈜엔에이치에프제14호공공임대위탁관리부동산투자회사</t>
         </is>
       </c>
     </row>
     <row r="253">
       <c r="A253" t="inlineStr">
         <is>
-          <t>㈜민간임대허브제5호위탁관리부동산투자회사</t>
+          <t>㈜엔에이치에프제15호공공임대위탁관리부동산투자회사</t>
         </is>
       </c>
     </row>
     <row r="254">
       <c r="A254" t="inlineStr">
         <is>
-          <t>㈜민간임대허브제6호위탁관리부동산투자회사</t>
+          <t>㈜엔에이치에프제1호공공임대위탁관리부동산투자회사</t>
         </is>
       </c>
     </row>
     <row r="255">
       <c r="A255" t="inlineStr">
         <is>
-          <t>㈜민간임대허브제7호위탁관리부동산투자회사</t>
+          <t>㈜엔에이치에프제2호공공임대위탁관리부동산투자회사</t>
         </is>
       </c>
     </row>
     <row r="256">
       <c r="A256" t="inlineStr">
         <is>
-          <t>㈜민간임대허브제8호위탁관리부동산투자회사</t>
+          <t>㈜엔에이치에프제3호공공임대위탁관리부동산투자회사</t>
         </is>
       </c>
     </row>
     <row r="257">
       <c r="A257" t="inlineStr">
         <is>
-          <t>㈜서울리츠임대주택제1호위탁관리부동산투자회사</t>
+          <t>㈜엔에이치에프제4호공공임대위탁관리부동산투자회사</t>
         </is>
       </c>
     </row>
     <row r="258">
       <c r="A258" t="inlineStr">
         <is>
-          <t>㈜서울사회주택토지지원위탁관리부동산투자회사</t>
+          <t>㈜엔에이치에프제5호공공임대위탁관리부동산투자회사</t>
         </is>
       </c>
     </row>
     <row r="259">
       <c r="A259" t="inlineStr">
         <is>
-          <t>㈜에스이그린에너지</t>
+          <t>㈜엔에이치에프제6호공공임대위탁관리부동산투자회사</t>
         </is>
       </c>
     </row>
     <row r="260">
       <c r="A260" t="inlineStr">
         <is>
-          <t>㈜에이치엘제2호위탁관리부동산투자회사</t>
+          <t>㈜엔에이치에프제7호공공임대위탁관리부동산투자회사</t>
         </is>
       </c>
     </row>
     <row r="261">
       <c r="A261" t="inlineStr">
         <is>
-          <t>㈜에이치엘제5호위탁관리부동산투자회사</t>
+          <t>㈜엔에이치에프제8호공공임대위탁관리부동산투자회사</t>
         </is>
       </c>
     </row>
     <row r="262">
       <c r="A262" t="inlineStr">
         <is>
-          <t>㈜에이팸</t>
+          <t>㈜엔에이치에프제9호공공임대위탁관리부동산투자회사</t>
         </is>
       </c>
     </row>
     <row r="263">
       <c r="A263" t="inlineStr">
         <is>
-          <t>㈜엔에이치에프제10호공공임대위탁관리부동산투자회사</t>
+          <t>㈜예미지뉴스테이기업형임대위탁관리부동산투자회사</t>
         </is>
       </c>
     </row>
     <row r="264">
       <c r="A264" t="inlineStr">
         <is>
-          <t>㈜엔에이치에프제11호공공임대위탁관리부동산투자회사</t>
+          <t>㈜우리천안두정위탁관리부동산투자회사</t>
         </is>
       </c>
     </row>
     <row r="265">
       <c r="A265" t="inlineStr">
         <is>
-          <t>㈜엔에이치에프제12호공공임대위탁관리부동산투자회사</t>
+          <t>㈜위례뉴스테이기업형임대위탁관리부동산투자회사</t>
         </is>
       </c>
     </row>
     <row r="266">
       <c r="A266" t="inlineStr">
         <is>
-          <t>㈜엔에이치에프제13호공공임대위탁관리부동산투자회사</t>
+          <t>㈜인천도화공공임대위탁관리부동산투자회사</t>
         </is>
       </c>
     </row>
     <row r="267">
       <c r="A267" t="inlineStr">
         <is>
-          <t>㈜엔에이치에프제14호공공임대위탁관리부동산투자회사</t>
+          <t>㈜인천도화뉴스테이기업형임대위탁관리부동산투자회사</t>
         </is>
       </c>
     </row>
     <row r="268">
       <c r="A268" t="inlineStr">
         <is>
-          <t>㈜엔에이치에프제15호공공임대위탁관리부동산투자회사</t>
+          <t>㈜인천도화위탁관리부동산투자회사</t>
         </is>
       </c>
     </row>
     <row r="269">
       <c r="A269" t="inlineStr">
         <is>
-          <t>㈜엔에이치에프제1호공공임대위탁관리부동산투자회사</t>
+          <t>㈜조흥포장</t>
         </is>
       </c>
     </row>
     <row r="270">
       <c r="A270" t="inlineStr">
         <is>
-          <t>㈜엔에이치에프제2호공공임대위탁관리부동산투자회사</t>
+          <t>㈜청년희망임대주택위탁관리부동산투자회사</t>
         </is>
       </c>
     </row>
     <row r="271">
       <c r="A271" t="inlineStr">
         <is>
-          <t>㈜엔에이치에프제3호공공임대위탁관리부동산투자회사</t>
+          <t>㈜캠코씨에스</t>
         </is>
       </c>
     </row>
     <row r="272">
       <c r="A272" t="inlineStr">
         <is>
-          <t>㈜엔에이치에프제4호공공임대위탁관리부동산투자회사</t>
+          <t>㈜캠코에프엠씨</t>
         </is>
       </c>
     </row>
     <row r="273">
       <c r="A273" t="inlineStr">
         <is>
-          <t>㈜엔에이치에프제5호공공임대위탁관리부동산투자회사</t>
+          <t>㈜케이솔라신안</t>
         </is>
       </c>
     </row>
     <row r="274">
       <c r="A274" t="inlineStr">
         <is>
-          <t>㈜엔에이치에프제6호공공임대위탁관리부동산투자회사</t>
+          <t>㈜케이원제16호분당위탁관리부동산투자회사</t>
         </is>
       </c>
     </row>
     <row r="275">
       <c r="A275" t="inlineStr">
         <is>
-          <t>㈜엔에이치에프제7호공공임대위탁관리부동산투자회사</t>
+          <t>㈜코시트</t>
         </is>
       </c>
     </row>
     <row r="276">
       <c r="A276" t="inlineStr">
         <is>
-          <t>㈜엔에이치에프제8호공공임대위탁관리부동산투자회사</t>
+          <t>㈜콤스코시큐리티</t>
         </is>
       </c>
     </row>
     <row r="277">
       <c r="A277" t="inlineStr">
         <is>
-          <t>㈜엔에이치에프제9호공공임대위탁관리부동산투자회사</t>
+          <t>㈜콤스코투게더</t>
         </is>
       </c>
     </row>
     <row r="278">
       <c r="A278" t="inlineStr">
         <is>
-          <t>㈜예미지뉴스테이기업형임대위탁관리부동산투자회사</t>
+          <t>㈜토지지원리츠제2호위탁관리부동산투자회사</t>
         </is>
       </c>
     </row>
     <row r="279">
       <c r="A279" t="inlineStr">
         <is>
-          <t>㈜우리천안두정위탁관리부동산투자회사</t>
+          <t>㈜페타미디어</t>
         </is>
       </c>
     </row>
     <row r="280">
       <c r="A280" t="inlineStr">
         <is>
-          <t>㈜위례뉴스테이기업형임대위탁관리부동산투자회사</t>
+          <t>㈜펨코제7호민간임대주택위탁관리부동산투자회사</t>
         </is>
       </c>
     </row>
     <row r="281">
       <c r="A281" t="inlineStr">
         <is>
-          <t>㈜인천도화공공임대위탁관리부동산투자회사</t>
+          <t>㈜하나스테이제1호위탁관리부동산투자회사</t>
         </is>
       </c>
     </row>
     <row r="282">
       <c r="A282" t="inlineStr">
         <is>
-          <t>㈜인천도화뉴스테이기업형임대위탁관리부동산투자회사</t>
+          <t>㈜하나트러스트제8호위탁관리부동산투자회사</t>
         </is>
       </c>
     </row>
     <row r="283">
       <c r="A283" t="inlineStr">
         <is>
-          <t>㈜인천도화위탁관리부동산투자회사</t>
+          <t>㈜해피투게더스테이제1호위탁관리부동산투자회사</t>
         </is>
       </c>
     </row>
     <row r="284">
       <c r="A284" t="inlineStr">
         <is>
-          <t>㈜조흥포장</t>
+          <t>강릉영동대학교행복기숙사유한회사</t>
         </is>
       </c>
     </row>
     <row r="285">
       <c r="A285" t="inlineStr">
         <is>
-          <t>㈜청년희망임대주택위탁관리부동산투자회사</t>
+          <t>경기그린에너지㈜</t>
         </is>
       </c>
     </row>
     <row r="286">
       <c r="A286" t="inlineStr">
         <is>
-          <t>㈜캠코씨에스</t>
+          <t>경기산업(주)</t>
         </is>
       </c>
     </row>
     <row r="287">
       <c r="A287" t="inlineStr">
         <is>
-          <t>㈜캠코에프엠씨</t>
+          <t>경북글로벌교류센터유한회사</t>
         </is>
       </c>
     </row>
     <row r="288">
       <c r="A288" t="inlineStr">
         <is>
-          <t>㈜케이솔라신안</t>
+          <t>경인여자대학교행복기숙사유한회사</t>
         </is>
       </c>
     </row>
     <row r="289">
       <c r="A289" t="inlineStr">
         <is>
-          <t>㈜케이원제16호분당위탁관리부동산투자회사</t>
+          <t>경주풍력발전(주)</t>
         </is>
       </c>
     </row>
     <row r="290">
       <c r="A290" t="inlineStr">
         <is>
-          <t>㈜코시트</t>
+          <t>경희대학교국제캠퍼스학생기숙사유한회사</t>
         </is>
       </c>
     </row>
     <row r="291">
       <c r="A291" t="inlineStr">
         <is>
-          <t>㈜콤스코시큐리티</t>
+          <t>경희대학교서울캠퍼스행복기숙사유한회사</t>
         </is>
       </c>
     </row>
     <row r="292">
       <c r="A292" t="inlineStr">
         <is>
-          <t>㈜콤스코투게더</t>
+          <t>고속도로태양광발전㈜</t>
         </is>
       </c>
     </row>
     <row r="293">
       <c r="A293" t="inlineStr">
         <is>
-          <t>㈜토지지원리츠제2호위탁관리부동산투자회사</t>
+          <t>고신대학교행복기숙사유한회사</t>
         </is>
       </c>
     </row>
     <row r="294">
       <c r="A294" t="inlineStr">
         <is>
-          <t>㈜페타미디어</t>
+          <t>광운대학교행복기숙사유한회사</t>
         </is>
       </c>
     </row>
     <row r="295">
       <c r="A295" t="inlineStr">
         <is>
-          <t>㈜펨코제7호민간임대주택위탁관리부동산투자회사</t>
+          <t>국제28호선박투자회사</t>
         </is>
       </c>
     </row>
     <row r="296">
       <c r="A296" t="inlineStr">
         <is>
-          <t>㈜하나스테이제1호위탁관리부동산투자회사</t>
+          <t>국제34호선박투자회사</t>
         </is>
       </c>
     </row>
     <row r="297">
       <c r="A297" t="inlineStr">
         <is>
-          <t>㈜하나트러스트제8호위탁관리부동산투자회사</t>
+          <t>국제35호선박투자회사</t>
         </is>
       </c>
     </row>
     <row r="298">
       <c r="A298" t="inlineStr">
         <is>
-          <t>㈜해피투게더스테이제1호위탁관리부동산투자회사</t>
+          <t>국제37호선박투자회사</t>
         </is>
       </c>
     </row>
     <row r="299">
       <c r="A299" t="inlineStr">
         <is>
-          <t>강릉영동대학교행복기숙사유한회사</t>
+          <t>국제41호선박투자회사</t>
         </is>
       </c>
     </row>
     <row r="300">
       <c r="A300" t="inlineStr">
         <is>
-          <t>경기그린에너지㈜</t>
+          <t>국제43호선박투자회사</t>
         </is>
       </c>
     </row>
     <row r="301">
       <c r="A301" t="inlineStr">
         <is>
-          <t>경기산업(주)</t>
+          <t>국제44호선박투자회사</t>
         </is>
       </c>
     </row>
     <row r="302">
       <c r="A302" t="inlineStr">
         <is>
-          <t>경북글로벌교류센터유한회사</t>
+          <t>국제45호선박투자회사</t>
         </is>
       </c>
     </row>
     <row r="303">
       <c r="A303" t="inlineStr">
         <is>
-          <t>경인여자대학교행복기숙사유한회사</t>
+          <t>국제46호선박투자회사</t>
         </is>
       </c>
     </row>
     <row r="304">
       <c r="A304" t="inlineStr">
         <is>
-          <t>경주풍력발전(주)</t>
+          <t>국제47호선박투자회사</t>
         </is>
       </c>
     </row>
     <row r="305">
       <c r="A305" t="inlineStr">
         <is>
-          <t>경희대학교국제캠퍼스학생기숙사유한회사</t>
+          <t>국제49호선박투자회사</t>
         </is>
       </c>
     </row>
     <row r="306">
       <c r="A306" t="inlineStr">
         <is>
-          <t>경희대학교서울캠퍼스행복기숙사유한회사</t>
+          <t>국제통신(주)</t>
         </is>
       </c>
     </row>
     <row r="307">
       <c r="A307" t="inlineStr">
         <is>
-          <t>고속도로태양광발전㈜</t>
+          <t>그랜드코리아레저(주)</t>
         </is>
       </c>
     </row>
     <row r="308">
       <c r="A308" t="inlineStr">
         <is>
-          <t>고신대학교행복기숙사유한회사</t>
+          <t>극동대학교행복기숙사유한회사</t>
         </is>
       </c>
     </row>
     <row r="309">
       <c r="A309" t="inlineStr">
         <is>
-          <t>광운대학교행복기숙사유한회사</t>
+          <t>기술금융제일호사모투자전문회사</t>
         </is>
       </c>
     </row>
     <row r="310">
       <c r="A310" t="inlineStr">
         <is>
-          <t>국제28호선박투자회사</t>
+          <t>기업구조혁신사모투자합자회사4호</t>
         </is>
       </c>
     </row>
     <row r="311">
       <c r="A311" t="inlineStr">
         <is>
-          <t>국제34호선박투자회사</t>
+          <t>기업구조혁신재정사모투자합자회사5호</t>
         </is>
       </c>
     </row>
     <row r="312">
       <c r="A312" t="inlineStr">
         <is>
-          <t>국제35호선박투자회사</t>
+          <t>기업구조혁신재정사모투자합자회사6호</t>
         </is>
       </c>
     </row>
     <row r="313">
       <c r="A313" t="inlineStr">
         <is>
-          <t>국제37호선박투자회사</t>
+          <t>기업구조혁신정책사모투자합자회사5호</t>
         </is>
       </c>
     </row>
     <row r="314">
       <c r="A314" t="inlineStr">
         <is>
-          <t>국제41호선박투자회사</t>
+          <t>기업구조혁신정책사모투자합자회사6호</t>
         </is>
       </c>
     </row>
     <row r="315">
       <c r="A315" t="inlineStr">
         <is>
-          <t>국제43호선박투자회사</t>
+          <t>기업은행(중국)유한공사</t>
         </is>
       </c>
     </row>
     <row r="316">
       <c r="A316" t="inlineStr">
         <is>
-          <t>국제44호선박투자회사</t>
+          <t>김포공항및주변지역개발사업주식회사</t>
         </is>
       </c>
     </row>
     <row r="317">
       <c r="A317" t="inlineStr">
         <is>
-          <t>국제45호선박투자회사</t>
+          <t>나사렛대학교행복기숙사유한회사</t>
         </is>
       </c>
     </row>
     <row r="318">
       <c r="A318" t="inlineStr">
         <is>
-          <t>국제46호선박투자회사</t>
+          <t>남부공항서비스주식회사</t>
         </is>
       </c>
     </row>
     <row r="319">
       <c r="A319" t="inlineStr">
         <is>
-          <t>국제47호선박투자회사</t>
+          <t>노앤자원순환제1호사모투자합자회사</t>
         </is>
       </c>
     </row>
     <row r="320">
       <c r="A320" t="inlineStr">
         <is>
-          <t>국제49호선박투자회사</t>
+          <t>단국대학교행복기숙사유한회사</t>
         </is>
       </c>
     </row>
     <row r="321">
       <c r="A321" t="inlineStr">
         <is>
-          <t>국제통신(주)</t>
+          <t>대경대학교행복기숙사유한회사</t>
         </is>
       </c>
     </row>
     <row r="322">
       <c r="A322" t="inlineStr">
         <is>
-          <t>그랜드코리아레저(주)</t>
+          <t>대구한의대학교행복기숙사유한회사</t>
         </is>
       </c>
     </row>
     <row r="323">
       <c r="A323" t="inlineStr">
         <is>
-          <t>그린이니셔티브2호사모투자합자회사</t>
+          <t>대전보건대학교행복기숙사유한회사</t>
         </is>
       </c>
     </row>
     <row r="324">
       <c r="A324" t="inlineStr">
         <is>
-          <t>극동대학교행복기숙사유한회사</t>
+          <t>대진대학교행복기숙사유한회사</t>
         </is>
       </c>
     </row>
     <row r="325">
       <c r="A325" t="inlineStr">
         <is>
-          <t>기술금융제일호사모투자전문회사</t>
+          <t>도로교통안전관리주식회사</t>
         </is>
       </c>
     </row>
     <row r="326">
       <c r="A326" t="inlineStr">
         <is>
-          <t>기업구조혁신사모투자합자회사4호</t>
+          <t>동남보건대학교행복기숙사유한회사</t>
         </is>
       </c>
     </row>
     <row r="327">
       <c r="A327" t="inlineStr">
         <is>
-          <t>기업구조혁신재정사모투자합자회사5호</t>
+          <t>동해부유식해상풍력발전㈜</t>
         </is>
       </c>
     </row>
     <row r="328">
       <c r="A328" t="inlineStr">
         <is>
-          <t>기업구조혁신재정사모투자합자회사6호</t>
+          <t>드림비전스(주)</t>
         </is>
       </c>
     </row>
     <row r="329">
       <c r="A329" t="inlineStr">
         <is>
-          <t>기업구조혁신정책사모투자합자회사5호</t>
+          <t>디지털혁신성장펀드</t>
         </is>
       </c>
     </row>
     <row r="330">
       <c r="A330" t="inlineStr">
         <is>
-          <t>기업구조혁신정책사모투자합자회사6호</t>
+          <t>베스람코리아(주)</t>
         </is>
       </c>
     </row>
     <row r="331">
       <c r="A331" t="inlineStr">
         <is>
-          <t>기업유동성지원기구</t>
+          <t>베이징KIDP산업디자인서비스유한공사</t>
         </is>
       </c>
     </row>
     <row r="332">
       <c r="A332" t="inlineStr">
         <is>
-          <t>기업은행(중국)유한공사</t>
+          <t>부산울산고속도로</t>
         </is>
       </c>
     </row>
     <row r="333">
       <c r="A333" t="inlineStr">
         <is>
-          <t>김포공항및주변지역개발사업주식회사</t>
+          <t>북경한능환보기술자문유한공사</t>
         </is>
       </c>
     </row>
     <row r="334">
       <c r="A334" t="inlineStr">
         <is>
-          <t>나사렛대학교행복기숙사유한회사</t>
+          <t>브랜드케이청년창조기술금융사모투자합자회사</t>
         </is>
       </c>
     </row>
     <row r="335">
       <c r="A335" t="inlineStr">
         <is>
-          <t>남부공항서비스주식회사</t>
+          <t>비전소재부품장비벤처투자조합제1호((주)리비콘에대한투자)</t>
         </is>
       </c>
     </row>
     <row r="336">
       <c r="A336" t="inlineStr">
         <is>
-          <t>노앤자원순환제1호사모투자합자회사</t>
+          <t>상명대학교행복기숙사유한회사</t>
         </is>
       </c>
     </row>
     <row r="337">
       <c r="A337" t="inlineStr">
         <is>
-          <t>단국대학교행복기숙사유한회사</t>
+          <t>상지대학교행복기숙사유한회사</t>
         </is>
       </c>
     </row>
     <row r="338">
       <c r="A338" t="inlineStr">
         <is>
-          <t>대경대학교행복기숙사유한회사</t>
+          <t>서부발전창기태양광(주)(구,삼양태양광(주))</t>
         </is>
       </c>
     </row>
     <row r="339">
       <c r="A339" t="inlineStr">
         <is>
-          <t>대구한의대학교행복기숙사유한회사</t>
+          <t>서영대학교행복기숙사유한회사</t>
         </is>
       </c>
     </row>
     <row r="340">
       <c r="A340" t="inlineStr">
         <is>
-          <t>대전보건대학교행복기숙사유한회사</t>
+          <t>서울보증보험(주)</t>
         </is>
       </c>
     </row>
     <row r="341">
       <c r="A341" t="inlineStr">
         <is>
-          <t>대진대학교행복기숙사유한회사</t>
+          <t>성공회대학교행복기숙사유한회사</t>
         </is>
       </c>
     </row>
     <row r="342">
       <c r="A342" t="inlineStr">
         <is>
-          <t>도로교통안전관리주식회사</t>
+          <t>성민산업(주)</t>
         </is>
       </c>
     </row>
     <row r="343">
       <c r="A343" t="inlineStr">
         <is>
-          <t>동남보건대학교행복기숙사유한회사</t>
+          <t>세종대학교행복기숙사유한회사</t>
         </is>
       </c>
     </row>
     <row r="344">
       <c r="A344" t="inlineStr">
         <is>
-          <t>동해부유식해상풍력발전㈜</t>
+          <t>송원대학교행복기숙사유한회사</t>
         </is>
       </c>
     </row>
     <row r="345">
       <c r="A345" t="inlineStr">
         <is>
-          <t>드림비전스(주)</t>
+          <t>수성대학교행복기숙사유한회사</t>
         </is>
       </c>
     </row>
     <row r="346">
       <c r="A346" t="inlineStr">
         <is>
-          <t>디지털혁신성장펀드</t>
+          <t>수은베트남리스금융회사</t>
         </is>
       </c>
     </row>
     <row r="347">
       <c r="A347" t="inlineStr">
         <is>
-          <t>베스람코리아(주)</t>
+          <t>수은싱가포르</t>
         </is>
       </c>
     </row>
     <row r="348">
       <c r="A348" t="inlineStr">
         <is>
-          <t>베이징KIDP산업디자인서비스유한공사</t>
+          <t>수은아주금융유한공사</t>
         </is>
       </c>
     </row>
     <row r="349">
       <c r="A349" t="inlineStr">
         <is>
-          <t>부산울산고속도로</t>
+          <t>수은영국은행</t>
         </is>
       </c>
     </row>
     <row r="350">
       <c r="A350" t="inlineStr">
         <is>
-          <t>북경한능환보기술자문유한공사</t>
+          <t>수은인니금융</t>
         </is>
       </c>
     </row>
     <row r="351">
       <c r="A351" t="inlineStr">
         <is>
-          <t>브랜드케이청년창조기술금융사모투자합자회사</t>
+          <t>수은플러스(주)</t>
         </is>
       </c>
     </row>
     <row r="352">
       <c r="A352" t="inlineStr">
         <is>
-          <t>블루오션기업재무안정제1호사모투자전문회사합자회사</t>
+          <t>스타트업코리아IBKVC-FP2024펀드</t>
         </is>
       </c>
     </row>
     <row r="353">
       <c r="A353" t="inlineStr">
         <is>
-          <t>비전소재부품장비벤처투자조합제1호((주)리비콘에대한투자)</t>
+          <t>스타트업코리아IBKVC-코오롱2024펀드</t>
         </is>
       </c>
     </row>
     <row r="354">
       <c r="A354" t="inlineStr">
         <is>
-          <t>산은비즈(주)</t>
+          <t>시큐텍㈜</t>
         </is>
       </c>
     </row>
     <row r="355">
       <c r="A355" t="inlineStr">
         <is>
-          <t>산은인베스트먼트(주)</t>
+          <t>신보글로벌2024제2차유동화전문회사(유)</t>
         </is>
       </c>
     </row>
     <row r="356">
       <c r="A356" t="inlineStr">
         <is>
-          <t>산은인프라자산운용(주)</t>
+          <t>신보운영관리(주)</t>
         </is>
       </c>
     </row>
     <row r="357">
       <c r="A357" t="inlineStr">
         <is>
-          <t>산은캐피탈(주)</t>
+          <t>신한대학교의정부캠퍼스행복기숙사유한회사</t>
         </is>
       </c>
     </row>
     <row r="358">
       <c r="A358" t="inlineStr">
         <is>
-          <t>상명대학교행복기숙사유한회사</t>
+          <t>아리랑TV미디어</t>
         </is>
       </c>
     </row>
     <row r="359">
       <c r="A359" t="inlineStr">
         <is>
-          <t>상지대학교행복기숙사유한회사</t>
+          <t>아이비케이금융그룹창공1호투자조합</t>
         </is>
       </c>
     </row>
     <row r="360">
       <c r="A360" t="inlineStr">
         <is>
-          <t>서부발전창기태양광(주)(구,삼양태양광(주))</t>
+          <t>아이비케이비엔더블유기술금융2018사모투자합자회사</t>
         </is>
       </c>
     </row>
     <row r="361">
       <c r="A361" t="inlineStr">
         <is>
-          <t>서영대학교행복기숙사유한회사</t>
+          <t>아이비케이비엔더블유산업경쟁력성장지원사모투자합자회사</t>
         </is>
       </c>
     </row>
     <row r="362">
       <c r="A362" t="inlineStr">
         <is>
-          <t>서울보증보험(주)</t>
+          <t>아이비케이스톤브릿지뉴딜이에스지유니콘사모투자합자회사</t>
         </is>
       </c>
     </row>
     <row r="363">
       <c r="A363" t="inlineStr">
         <is>
-          <t>성공회대학교행복기숙사유한회사</t>
+          <t>아이비케이스톤브릿지혁신성장사모투자합자회사</t>
         </is>
       </c>
     </row>
     <row r="364">
       <c r="A364" t="inlineStr">
         <is>
-          <t>성민산업(주)</t>
+          <t>아이비케이엘엑스지스케일업수출지원사모투자합자회사</t>
         </is>
       </c>
     </row>
     <row r="365">
       <c r="A365" t="inlineStr">
         <is>
-          <t>세종대학교행복기숙사유한회사</t>
+          <t>아이비케이케이아이피성장디딤돌제1호사모투자합자회사</t>
         </is>
       </c>
     </row>
     <row r="366">
       <c r="A366" t="inlineStr">
         <is>
-          <t>송원대학교행복기숙사유한회사</t>
+          <t>아이비케이키움사업재편사모투자합자회사</t>
         </is>
       </c>
     </row>
     <row r="367">
       <c r="A367" t="inlineStr">
         <is>
-          <t>수성대학교행복기숙사유한회사</t>
+          <t>아이비케이키움중소중견점프업사모투자합자회사</t>
         </is>
       </c>
     </row>
     <row r="368">
       <c r="A368" t="inlineStr">
         <is>
-          <t>수은베트남리스금융회사</t>
+          <t>아이비케이티에스엑시트제2호사모투자합자회사</t>
         </is>
       </c>
     </row>
     <row r="369">
       <c r="A369" t="inlineStr">
         <is>
-          <t>수은싱가포르</t>
+          <t>아이비케이포스코트루벤기업재무안정사모투자전문회사</t>
         </is>
       </c>
     </row>
     <row r="370">
       <c r="A370" t="inlineStr">
         <is>
-          <t>수은아주금융유한공사</t>
+          <t>아이비케이한국투자성장사다리사모투자합자회사</t>
         </is>
       </c>
     </row>
     <row r="371">
       <c r="A371" t="inlineStr">
         <is>
-          <t>수은영국은행</t>
+          <t>아주대학교행복기숙사유한회사</t>
         </is>
       </c>
     </row>
     <row r="372">
       <c r="A372" t="inlineStr">
         <is>
-          <t>수은인니금융</t>
+          <t>알이비파트너스주식회사</t>
         </is>
       </c>
     </row>
     <row r="373">
       <c r="A373" t="inlineStr">
         <is>
-          <t>수은플러스(주)</t>
+          <t>앨리스-하나에스앤비소부장신기술투자조합</t>
         </is>
       </c>
     </row>
     <row r="374">
       <c r="A374" t="inlineStr">
         <is>
-          <t>스마일게이트소재부품투자펀드2014-3호</t>
+          <t>양구수상태양광(주)</t>
         </is>
       </c>
     </row>
     <row r="375">
       <c r="A375" t="inlineStr">
         <is>
-          <t>스타트업코리아IBKVC-FP2024펀드</t>
+          <t>에너지신산업전문투자사모투자신탁</t>
         </is>
       </c>
     </row>
     <row r="376">
       <c r="A376" t="inlineStr">
         <is>
-          <t>스타트업코리아IBKVC-코오롱2024펀드</t>
+          <t>에너지혁신성장펀드1호</t>
         </is>
       </c>
     </row>
     <row r="377">
       <c r="A377" t="inlineStr">
         <is>
-          <t>시큐텍㈜</t>
+          <t>에듀이십일건국대기숙사유한회사</t>
         </is>
       </c>
     </row>
     <row r="378">
       <c r="A378" t="inlineStr">
         <is>
-          <t>신보글로벌2024제2차유동화전문회사(유)</t>
+          <t>에스비케이엘지엘사모투자합자회사</t>
         </is>
       </c>
     </row>
     <row r="379">
       <c r="A379" t="inlineStr">
         <is>
-          <t>신보운영관리(주)</t>
+          <t>에스비케이와스카사모투자합자회사</t>
         </is>
       </c>
     </row>
     <row r="380">
       <c r="A380" t="inlineStr">
         <is>
-          <t>신한대학교의정부캠퍼스행복기숙사유한회사</t>
+          <t>에스엠푸드(주)</t>
         </is>
       </c>
     </row>
     <row r="381">
       <c r="A381" t="inlineStr">
         <is>
-          <t>아리랑TV미디어</t>
+          <t>에이치에프파트너스주식회사</t>
         </is>
       </c>
     </row>
     <row r="382">
       <c r="A382" t="inlineStr">
         <is>
-          <t>아세안바이오메디컬투자조합</t>
+          <t>에이플(주)</t>
         </is>
       </c>
     </row>
     <row r="383">
       <c r="A383" t="inlineStr">
         <is>
-          <t>아이비케이금융그룹창공1호투자조합</t>
+          <t>엔에스엘이디(주)</t>
         </is>
       </c>
     </row>
     <row r="384">
       <c r="A384" t="inlineStr">
         <is>
-          <t>아이비케이비엔더블유기술금융2018사모투자합자회사</t>
+          <t>엘에이치주거복지정보(주)</t>
         </is>
       </c>
     </row>
     <row r="385">
       <c r="A385" t="inlineStr">
         <is>
-          <t>아이비케이비엔더블유산업경쟁력성장지원사모투자합자회사</t>
+          <t>엘엑스파트너스(주)</t>
         </is>
       </c>
     </row>
     <row r="386">
       <c r="A386" t="inlineStr">
         <is>
-          <t>아이비케이스톤브릿지뉴딜이에스지유니콘사모투자합자회사</t>
+          <t>엠티솔루션경서판매(주)</t>
         </is>
       </c>
     </row>
     <row r="387">
       <c r="A387" t="inlineStr">
         <is>
-          <t>아이비케이스톤브릿지혁신성장사모투자합자회사</t>
+          <t>여수광양항만관리(주)</t>
         </is>
       </c>
     </row>
     <row r="388">
       <c r="A388" t="inlineStr">
         <is>
-          <t>아이비케이에스중소기업도약사모투자합자회사</t>
+          <t>여수엑스포관리(주)</t>
         </is>
       </c>
     </row>
     <row r="389">
       <c r="A389" t="inlineStr">
         <is>
-          <t>아이비케이엘엑스지스케일업수출지원사모투자합자회사</t>
+          <t>영남이공대학교행복기숙사유한회사</t>
         </is>
       </c>
     </row>
     <row r="390">
       <c r="A390" t="inlineStr">
         <is>
-          <t>아이비케이케이아이피성장디딤돌제1호사모투자합자회사</t>
+          <t>영덕해맞이풍력(주)</t>
         </is>
       </c>
     </row>
     <row r="391">
       <c r="A391" t="inlineStr">
         <is>
-          <t>아이비케이키움사업재편사모투자합자회사</t>
+          <t>예별손해보험(주)</t>
         </is>
       </c>
     </row>
     <row r="392">
       <c r="A392" t="inlineStr">
         <is>
-          <t>아이비케이키움중소중견점프업사모투자합자회사</t>
+          <t>오기리태양광발전㈜</t>
         </is>
       </c>
     </row>
     <row r="393">
       <c r="A393" t="inlineStr">
         <is>
-          <t>아이비케이티에스엑시트제2호사모투자합자회사</t>
+          <t>온기업1호기업재무안정사모투자합자회사</t>
         </is>
       </c>
     </row>
     <row r="394">
       <c r="A394" t="inlineStr">
         <is>
-          <t>아이비케이포스코트루벤기업재무안정사모투자전문회사</t>
+          <t>용인대학교행복기숙사유한회사</t>
         </is>
       </c>
     </row>
     <row r="395">
       <c r="A395" t="inlineStr">
         <is>
-          <t>아이비케이한국투자성장사다리사모투자합자회사</t>
+          <t>우리전선(주)</t>
         </is>
       </c>
     </row>
     <row r="396">
       <c r="A396" t="inlineStr">
         <is>
-          <t>아주대학교행복기숙사유한회사</t>
+          <t>울산항만관리(주)</t>
         </is>
       </c>
     </row>
     <row r="397">
       <c r="A397" t="inlineStr">
         <is>
-          <t>알바트로스퓨처코리아투자조합</t>
+          <t>원광보건대학교행복기숙사유한회사</t>
         </is>
       </c>
     </row>
     <row r="398">
       <c r="A398" t="inlineStr">
         <is>
-          <t>알이비파트너스주식회사</t>
+          <t>원전산업성장펀드</t>
         </is>
       </c>
     </row>
     <row r="399">
       <c r="A399" t="inlineStr">
         <is>
-          <t>앨리스-하나에스앤비소부장신기술투자조합</t>
+          <t>이더블유피서비스(주)</t>
         </is>
       </c>
     </row>
     <row r="400">
       <c r="A400" t="inlineStr">
         <is>
-          <t>양구수상태양광(주)</t>
+          <t>이에이에스제오차유동화전문유한회사</t>
         </is>
       </c>
     </row>
     <row r="401">
       <c r="A401" t="inlineStr">
         <is>
-          <t>에너지신산업전문투자사모투자신탁</t>
+          <t>이지케어텍</t>
         </is>
       </c>
     </row>
     <row r="402">
       <c r="A402" t="inlineStr">
         <is>
-          <t>에너지혁신성장펀드1호</t>
+          <t>이지케어텍(주)</t>
         </is>
       </c>
     </row>
     <row r="403">
       <c r="A403" t="inlineStr">
         <is>
-          <t>에듀이십일건국대기숙사유한회사</t>
+          <t>익산글로벌교류센터유한회사</t>
         </is>
       </c>
     </row>
     <row r="404">
       <c r="A404" t="inlineStr">
         <is>
-          <t>에스비케이엘지엘사모투자합자회사</t>
+          <t>인비전사모투자합자회사</t>
         </is>
       </c>
     </row>
     <row r="405">
       <c r="A405" t="inlineStr">
         <is>
-          <t>에스비케이와스카사모투자합자회사</t>
+          <t>인천공항시설관리(주)</t>
         </is>
       </c>
     </row>
     <row r="406">
       <c r="A406" t="inlineStr">
         <is>
-          <t>에스엠푸드(주)</t>
+          <t>인천공항에너지(주)</t>
         </is>
       </c>
     </row>
     <row r="407">
       <c r="A407" t="inlineStr">
         <is>
-          <t>에이치에프파트너스주식회사</t>
+          <t>인천공항운영서비스(주)</t>
         </is>
       </c>
     </row>
     <row r="408">
       <c r="A408" t="inlineStr">
         <is>
-          <t>에이플(주)</t>
+          <t>인천국제공항보안(주)</t>
         </is>
       </c>
     </row>
     <row r="409">
       <c r="A409" t="inlineStr">
         <is>
-          <t>엔베스터창해유주사모투자합자회사</t>
+          <t>인천연료전지㈜</t>
         </is>
       </c>
     </row>
     <row r="410">
       <c r="A410" t="inlineStr">
         <is>
-          <t>엔에스엘이디(주)</t>
+          <t>인천항보안공사</t>
         </is>
       </c>
     </row>
     <row r="411">
       <c r="A411" t="inlineStr">
         <is>
-          <t>엔에이치엘비그로쓰챔프2011의4호사모투자전문회사합자회사</t>
+          <t>인하대학교행복기숙사유한회사</t>
         </is>
       </c>
     </row>
     <row r="412">
       <c r="A412" t="inlineStr">
         <is>
-          <t>엘에이치주거복지정보(주)</t>
+          <t>일품푸드(주)</t>
         </is>
       </c>
     </row>
     <row r="413">
       <c r="A413" t="inlineStr">
         <is>
-          <t>엘엑스파트너스(주)</t>
+          <t>임하수상태양광(주)</t>
         </is>
       </c>
     </row>
     <row r="414">
       <c r="A414" t="inlineStr">
         <is>
-          <t>엠티솔루션경서판매(주)</t>
+          <t>전주비전대학교행복기숙사유한회사</t>
         </is>
       </c>
     </row>
     <row r="415">
       <c r="A415" t="inlineStr">
         <is>
-          <t>여수광양항만관리(주)</t>
+          <t>정암풍력발전(주)</t>
         </is>
       </c>
     </row>
     <row r="416">
       <c r="A416" t="inlineStr">
         <is>
-          <t>여수엑스포관리(주)</t>
+          <t>제이디씨예래리조트(주)</t>
         </is>
       </c>
     </row>
     <row r="417">
       <c r="A417" t="inlineStr">
         <is>
-          <t>영남이공대학교행복기숙사유한회사</t>
+          <t>제이디씨파트너스(주)</t>
         </is>
       </c>
     </row>
     <row r="418">
       <c r="A418" t="inlineStr">
         <is>
-          <t>영덕해맞이풍력(주)</t>
+          <t>제주관광대학교행복기숙사유한회사</t>
         </is>
       </c>
     </row>
     <row r="419">
       <c r="A419" t="inlineStr">
         <is>
-          <t>예별손해보험(주)</t>
+          <t>제주한림해상풍력(주)</t>
         </is>
       </c>
     </row>
     <row r="420">
       <c r="A420" t="inlineStr">
         <is>
-          <t>오기리태양광발전㈜</t>
+          <t>주식회사 메디밸리파트너스</t>
         </is>
       </c>
     </row>
     <row r="421">
       <c r="A421" t="inlineStr">
         <is>
-          <t>온기업1호기업재무안정사모투자합자회사</t>
+          <t>주식회사 신아에스비(SLS조선)</t>
         </is>
       </c>
     </row>
     <row r="422">
       <c r="A422" t="inlineStr">
         <is>
-          <t>와이제이에이중소중견기업엠앤에이사모투자합자회사</t>
+          <t>주식회사 에버조이</t>
         </is>
       </c>
     </row>
     <row r="423">
       <c r="A423" t="inlineStr">
         <is>
-          <t>용인대학교행복기숙사유한회사</t>
+          <t>주식회사 에이디디보안환경관리단</t>
         </is>
       </c>
     </row>
     <row r="424">
       <c r="A424" t="inlineStr">
         <is>
-          <t>우리전선(주)</t>
+          <t>주식회사 에이디디시설관리단</t>
         </is>
       </c>
     </row>
     <row r="425">
       <c r="A425" t="inlineStr">
         <is>
-          <t>울산항만관리(주)</t>
+          <t>주택관리공단(주)</t>
         </is>
       </c>
     </row>
     <row r="426">
       <c r="A426" t="inlineStr">
         <is>
-          <t>원광보건대학교행복기숙사유한회사</t>
+          <t>주택도시보증공사(주택도시기금)</t>
         </is>
       </c>
     </row>
     <row r="427">
       <c r="A427" t="inlineStr">
         <is>
-          <t>원익그로쓰챔프2011의3호사모투자전문회사합자회사</t>
+          <t>중부발전서비스㈜</t>
         </is>
       </c>
     </row>
     <row r="428">
       <c r="A428" t="inlineStr">
         <is>
-          <t>원전산업성장펀드</t>
+          <t>중진공파트너스(주)</t>
         </is>
       </c>
     </row>
     <row r="429">
       <c r="A429" t="inlineStr">
         <is>
-          <t>웨일제1호중소중견기업엠앤에이사모투자합자회사</t>
+          <t>지성에스이(주)</t>
         </is>
       </c>
     </row>
     <row r="430">
       <c r="A430" t="inlineStr">
         <is>
-          <t>유안타세컨더리2호펀드</t>
+          <t>지엠에프구호선박투자회사</t>
         </is>
       </c>
     </row>
     <row r="431">
       <c r="A431" t="inlineStr">
         <is>
-          <t>이더블유피서비스(주)</t>
+          <t>지엠에프비비씨이호선박투자회사</t>
         </is>
       </c>
     </row>
     <row r="432">
       <c r="A432" t="inlineStr">
         <is>
-          <t>이에이에스제오차유동화전문유한회사</t>
+          <t>지엠에프비비씨일호선박투자회사</t>
         </is>
       </c>
     </row>
     <row r="433">
       <c r="A433" t="inlineStr">
         <is>
-          <t>이지케어텍</t>
+          <t>지엠에프삼호선박투자회사</t>
         </is>
       </c>
     </row>
     <row r="434">
       <c r="A434" t="inlineStr">
         <is>
-          <t>이지케어텍(주)</t>
+          <t>지엠에프십구호선박투자회사</t>
         </is>
       </c>
     </row>
     <row r="435">
       <c r="A435" t="inlineStr">
         <is>
-          <t>익산글로벌교류센터유한회사</t>
+          <t>지엠에프십사호선박투자회사</t>
         </is>
       </c>
     </row>
     <row r="436">
       <c r="A436" t="inlineStr">
         <is>
-          <t>인비전사모투자합자회사</t>
+          <t>지엠에프십삼호선박투자회사</t>
         </is>
       </c>
     </row>
     <row r="437">
       <c r="A437" t="inlineStr">
         <is>
-          <t>인천공항시설관리(주)</t>
+          <t>지엠에프십오호선박투자회사</t>
         </is>
       </c>
     </row>
     <row r="438">
       <c r="A438" t="inlineStr">
         <is>
-          <t>인천공항에너지(주)</t>
+          <t>지엠에프십육호선박투자회사</t>
         </is>
       </c>
     </row>
     <row r="439">
       <c r="A439" t="inlineStr">
         <is>
-          <t>인천공항운영서비스(주)</t>
+          <t>지엠에프십이호선박투자회사</t>
         </is>
       </c>
     </row>
     <row r="440">
       <c r="A440" t="inlineStr">
         <is>
-          <t>인천국제공항보안(주)</t>
+          <t>지엠에프십일호선박투자회사</t>
         </is>
       </c>
     </row>
     <row r="441">
       <c r="A441" t="inlineStr">
         <is>
-          <t>인천연료전지㈜</t>
+          <t>지엠에프십칠호선박투자회사</t>
         </is>
       </c>
     </row>
     <row r="442">
       <c r="A442" t="inlineStr">
         <is>
-          <t>인천항보안공사</t>
+          <t>지엠에프십팔호선박투자회사</t>
         </is>
       </c>
     </row>
     <row r="443">
       <c r="A443" t="inlineStr">
         <is>
-          <t>인하대학교행복기숙사유한회사</t>
+          <t>지엠에프십호선박투자회사</t>
         </is>
       </c>
     </row>
     <row r="444">
       <c r="A444" t="inlineStr">
         <is>
-          <t>일품푸드(주)</t>
+          <t>지엠에프육호선박투자회사</t>
         </is>
       </c>
     </row>
     <row r="445">
       <c r="A445" t="inlineStr">
         <is>
-          <t>임하수상태양광(주)</t>
+          <t>지엠에프이십사호선박투자회사</t>
         </is>
       </c>
     </row>
     <row r="446">
       <c r="A446" t="inlineStr">
         <is>
-          <t>전주비전대학교행복기숙사유한회사</t>
+          <t>지엠에프이십삼호선박투자회사</t>
         </is>
       </c>
     </row>
     <row r="447">
       <c r="A447" t="inlineStr">
         <is>
-          <t>정암풍력발전(주)</t>
+          <t>지엠에프이십육호선박투자회사</t>
         </is>
       </c>
     </row>
     <row r="448">
       <c r="A448" t="inlineStr">
         <is>
-          <t>제이디씨예래리조트(주)</t>
+          <t>지엠에프이십이호선박투자회사</t>
         </is>
       </c>
     </row>
     <row r="449">
       <c r="A449" t="inlineStr">
         <is>
-          <t>제이디씨파트너스(주)</t>
+          <t>지엠에프이십일호선박투자회사</t>
         </is>
       </c>
     </row>
     <row r="450">
       <c r="A450" t="inlineStr">
         <is>
-          <t>제주관광대학교행복기숙사유한회사</t>
+          <t>지엠에프이십칠호선박투자회사</t>
         </is>
       </c>
     </row>
     <row r="451">
       <c r="A451" t="inlineStr">
         <is>
-          <t>제주한림해상풍력(주)</t>
+          <t>지엠에프이십호선박투자회사</t>
         </is>
       </c>
     </row>
     <row r="452">
       <c r="A452" t="inlineStr">
         <is>
-          <t>주식회사 메디밸리파트너스</t>
+          <t>지엠에프이호선박투자회사</t>
         </is>
       </c>
     </row>
     <row r="453">
       <c r="A453" t="inlineStr">
         <is>
-          <t>주식회사 신아에스비(SLS조선)</t>
+          <t>지엠에프일호선박투자회사</t>
         </is>
       </c>
     </row>
     <row r="454">
       <c r="A454" t="inlineStr">
         <is>
-          <t>주식회사 에버조이</t>
+          <t>지엠에프칠호선박투자회사</t>
         </is>
       </c>
     </row>
     <row r="455">
       <c r="A455" t="inlineStr">
         <is>
-          <t>주식회사 에이디디보안환경관리단</t>
+          <t>지역난방안전(주)</t>
         </is>
       </c>
     </row>
     <row r="456">
       <c r="A456" t="inlineStr">
         <is>
-          <t>주식회사 에이디디시설관리단</t>
+          <t>지역난방플러스(주)</t>
         </is>
       </c>
     </row>
     <row r="457">
       <c r="A457" t="inlineStr">
         <is>
-          <t>주택관리공단(주)</t>
+          <t>지케이엘위드주식회사</t>
         </is>
       </c>
     </row>
     <row r="458">
       <c r="A458" t="inlineStr">
         <is>
-          <t>주택도시보증공사(주택도시기금)</t>
+          <t>찬우축산(주)</t>
         </is>
       </c>
     </row>
     <row r="459">
       <c r="A459" t="inlineStr">
         <is>
-          <t>중부발전서비스㈜</t>
+          <t>창죽풍력발전(주)</t>
         </is>
       </c>
     </row>
     <row r="460">
       <c r="A460" t="inlineStr">
         <is>
-          <t>중진공파트너스(주)</t>
+          <t>충북보건과학대학교행복기숙사유한회사</t>
         </is>
       </c>
     </row>
     <row r="461">
       <c r="A461" t="inlineStr">
         <is>
-          <t>지성에스이(주)</t>
+          <t>칭다오aT물류유한공사</t>
         </is>
       </c>
     </row>
     <row r="462">
       <c r="A462" t="inlineStr">
         <is>
-          <t>지엠에프구호선박투자회사</t>
+          <t>캠코기업지원금융㈜</t>
         </is>
       </c>
     </row>
     <row r="463">
       <c r="A463" t="inlineStr">
         <is>
-          <t>지엠에프비비씨이호선박투자회사</t>
+          <t>캠코동산금융지원㈜</t>
         </is>
       </c>
     </row>
     <row r="464">
       <c r="A464" t="inlineStr">
         <is>
-          <t>지엠에프비비씨일호선박투자회사</t>
+          <t>캠코선박운용㈜</t>
         </is>
       </c>
     </row>
     <row r="465">
       <c r="A465" t="inlineStr">
         <is>
-          <t>지엠에프삼호선박투자회사</t>
+          <t>케이바이오스타트</t>
         </is>
       </c>
     </row>
     <row r="466">
       <c r="A466" t="inlineStr">
         <is>
-          <t>지엠에프십구호선박투자회사</t>
+          <t>케이씨엘엔지테크(주)</t>
         </is>
       </c>
     </row>
     <row r="467">
       <c r="A467" t="inlineStr">
         <is>
-          <t>지엠에프십사호선박투자회사</t>
+          <t>케이앤에프파트너스(주)</t>
         </is>
       </c>
     </row>
     <row r="468">
       <c r="A468" t="inlineStr">
         <is>
-          <t>지엠에프십삼호선박투자회사</t>
+          <t>케이에스에프10호선박투자회사</t>
         </is>
       </c>
     </row>
     <row r="469">
       <c r="A469" t="inlineStr">
         <is>
-          <t>지엠에프십오호선박투자회사</t>
+          <t>케이에스에프11호선박투자회사</t>
         </is>
       </c>
     </row>
     <row r="470">
       <c r="A470" t="inlineStr">
         <is>
-          <t>지엠에프십육호선박투자회사</t>
+          <t>케이에스에프12호선박투자회사</t>
         </is>
       </c>
     </row>
     <row r="471">
       <c r="A471" t="inlineStr">
         <is>
-          <t>지엠에프십이호선박투자회사</t>
+          <t>케이에스에프17호선박투자회사</t>
         </is>
       </c>
     </row>
     <row r="472">
       <c r="A472" t="inlineStr">
         <is>
-          <t>지엠에프십일호선박투자회사</t>
+          <t>케이에스에프19호선박투자회사</t>
         </is>
       </c>
     </row>
     <row r="473">
       <c r="A473" t="inlineStr">
         <is>
-          <t>지엠에프십칠호선박투자회사</t>
+          <t>케이에스에프1호선박투자회사</t>
         </is>
       </c>
     </row>
     <row r="474">
       <c r="A474" t="inlineStr">
         <is>
-          <t>지엠에프십팔호선박투자회사</t>
+          <t>케이에스에프20호선박투자회사</t>
         </is>
       </c>
     </row>
     <row r="475">
       <c r="A475" t="inlineStr">
         <is>
-          <t>지엠에프십호선박투자회사</t>
+          <t>케이에스에프22호선박투자회사</t>
         </is>
       </c>
     </row>
     <row r="476">
       <c r="A476" t="inlineStr">
         <is>
-          <t>지엠에프육호선박투자회사</t>
+          <t>케이에스에프23호선박투자회사</t>
         </is>
       </c>
     </row>
     <row r="477">
       <c r="A477" t="inlineStr">
         <is>
-          <t>지엠에프이십사호선박투자회사</t>
+          <t>케이에스에프24호선박투자회사</t>
         </is>
       </c>
     </row>
     <row r="478">
       <c r="A478" t="inlineStr">
         <is>
-          <t>지엠에프이십삼호선박투자회사</t>
+          <t>케이에스에프26호선박투자회사</t>
         </is>
       </c>
     </row>
     <row r="479">
       <c r="A479" t="inlineStr">
         <is>
-          <t>지엠에프이십육호선박투자회사</t>
+          <t>케이에스에프27호선박투자회사</t>
         </is>
       </c>
     </row>
     <row r="480">
       <c r="A480" t="inlineStr">
         <is>
-          <t>지엠에프이십이호선박투자회사</t>
+          <t>케이에스에프28호선박투자회사</t>
         </is>
       </c>
     </row>
     <row r="481">
       <c r="A481" t="inlineStr">
         <is>
-          <t>지엠에프이십일호선박투자회사</t>
+          <t>케이에스에프29호선박투자회사</t>
         </is>
       </c>
     </row>
     <row r="482">
       <c r="A482" t="inlineStr">
         <is>
-          <t>지엠에프이십칠호선박투자회사</t>
+          <t>케이에스에프2호선박투자회사</t>
         </is>
       </c>
     </row>
     <row r="483">
       <c r="A483" t="inlineStr">
         <is>
-          <t>지엠에프이십호선박투자회사</t>
+          <t>케이에스에프30호선박투자회사</t>
         </is>
       </c>
     </row>
     <row r="484">
       <c r="A484" t="inlineStr">
         <is>
-          <t>지엠에프이호선박투자회사</t>
+          <t>케이에스에프31호선박투자회사</t>
         </is>
       </c>
     </row>
     <row r="485">
       <c r="A485" t="inlineStr">
         <is>
-          <t>지엠에프일호선박투자회사</t>
+          <t>케이에스에프32호선박투자회사</t>
         </is>
       </c>
     </row>
     <row r="486">
       <c r="A486" t="inlineStr">
         <is>
-          <t>지엠에프칠호선박투자회사</t>
+          <t>케이에스에프33호선박투자회사</t>
         </is>
       </c>
     </row>
     <row r="487">
       <c r="A487" t="inlineStr">
         <is>
-          <t>지역난방안전(주)</t>
+          <t>케이에스에프34호선박투자회사</t>
         </is>
       </c>
     </row>
     <row r="488">
       <c r="A488" t="inlineStr">
         <is>
-          <t>지역난방플러스(주)</t>
+          <t>케이에스에프35호선박투자회사</t>
         </is>
       </c>
     </row>
     <row r="489">
       <c r="A489" t="inlineStr">
         <is>
-          <t>지케이엘위드주식회사</t>
+          <t>케이에스에프36호선박투자회사</t>
         </is>
       </c>
     </row>
     <row r="490">
       <c r="A490" t="inlineStr">
         <is>
-          <t>찬우축산(주)</t>
+          <t>케이에스에프37호선박투자회사</t>
         </is>
       </c>
     </row>
     <row r="491">
       <c r="A491" t="inlineStr">
         <is>
-          <t>창죽풍력발전(주)</t>
+          <t>케이에스에프38호선박투자회사</t>
         </is>
       </c>
     </row>
     <row r="492">
       <c r="A492" t="inlineStr">
         <is>
-          <t>충북보건과학대학교행복기숙사유한회사</t>
+          <t>케이에스에프39호선박투자회사</t>
         </is>
       </c>
     </row>
     <row r="493">
       <c r="A493" t="inlineStr">
         <is>
-          <t>충청권글로벌기술투자조합</t>
+          <t>케이에스에프40호선박투자회사</t>
         </is>
       </c>
     </row>
     <row r="494">
       <c r="A494" t="inlineStr">
         <is>
-          <t>칭다오aT물류유한공사</t>
+          <t>케이에스에프41호선박투자회사</t>
         </is>
       </c>
     </row>
     <row r="495">
       <c r="A495" t="inlineStr">
         <is>
-          <t>캠코기업지원금융㈜</t>
+          <t>케이에스에프42호선박투자회사</t>
         </is>
       </c>
     </row>
     <row r="496">
       <c r="A496" t="inlineStr">
         <is>
-          <t>캠코동산금융지원㈜</t>
+          <t>케이에스에프43호선박투자회사</t>
         </is>
       </c>
     </row>
     <row r="497">
       <c r="A497" t="inlineStr">
         <is>
-          <t>캠코선박운용㈜</t>
+          <t>케이에스에프8호선박투자회사</t>
         </is>
       </c>
     </row>
     <row r="498">
       <c r="A498" t="inlineStr">
         <is>
-          <t>케이디비대성-HGI그린임팩트투자조합</t>
+          <t>케이에이씨공항서비스주식회사</t>
         </is>
       </c>
     </row>
     <row r="499">
       <c r="A499" t="inlineStr">
         <is>
-          <t>케이디비생명보험(주)</t>
+          <t>케이엔오씨서비스(주)</t>
         </is>
       </c>
     </row>
     <row r="500">
       <c r="A500" t="inlineStr">
         <is>
-          <t>케이디비아시아사모투자합자회사</t>
+          <t>케이워터기술(주)</t>
         </is>
       </c>
     </row>
     <row r="501">
       <c r="A501" t="inlineStr">
         <is>
-          <t>케이디비아이에이피일대일로사모투자합자회사</t>
+          <t>케이워터운영관리(주)</t>
         </is>
       </c>
     </row>
     <row r="502">
       <c r="A502" t="inlineStr">
         <is>
-          <t>케이디비아이하나사업재편밸류업사모투자합자회사</t>
+          <t>케이티오파트너스(주)</t>
         </is>
       </c>
     </row>
     <row r="503">
       <c r="A503" t="inlineStr">
         <is>
-          <t>케이디비중소중견메자닌사모투자합자회사</t>
+          <t>케이피에스파트너스㈜</t>
         </is>
       </c>
     </row>
     <row r="504">
       <c r="A504" t="inlineStr">
         <is>
-          <t>케이디비칸서스밸류사모투자전문회사</t>
+          <t>케이피엑스서비스원주식회사</t>
         </is>
       </c>
     </row>
     <row r="505">
       <c r="A505" t="inlineStr">
         <is>
-          <t>케이디비케이엘중소중견밸류업제2호사모투자(자)</t>
+          <t>켑코솔라(주)</t>
         </is>
       </c>
     </row>
     <row r="506">
       <c r="A506" t="inlineStr">
         <is>
-          <t>케이바이오스타트</t>
+          <t>켑코이에스(주)</t>
         </is>
       </c>
     </row>
     <row r="507">
       <c r="A507" t="inlineStr">
         <is>
-          <t>케이씨엘엔지테크(주)</t>
+          <t>코가스보안관리(주)(주6)</t>
         </is>
       </c>
     </row>
     <row r="508">
       <c r="A508" t="inlineStr">
         <is>
-          <t>케이앤에프파트너스(주)</t>
+          <t>코가스서비스얼라이언스(주)(주6)</t>
         </is>
       </c>
     </row>
     <row r="509">
       <c r="A509" t="inlineStr">
         <is>
-          <t>케이에스에프10호선박투자회사</t>
+          <t>코레일관광개발㈜</t>
         </is>
       </c>
     </row>
     <row r="510">
       <c r="A510" t="inlineStr">
         <is>
-          <t>케이에스에프11호선박투자회사</t>
+          <t>코레일네트웍스㈜</t>
         </is>
       </c>
     </row>
     <row r="511">
       <c r="A511" t="inlineStr">
         <is>
-          <t>케이에스에프12호선박투자회사</t>
+          <t>코레일로지스㈜</t>
         </is>
       </c>
     </row>
     <row r="512">
       <c r="A512" t="inlineStr">
         <is>
-          <t>케이에스에프17호선박투자회사</t>
+          <t>코레일유통㈜</t>
         </is>
       </c>
     </row>
     <row r="513">
       <c r="A513" t="inlineStr">
         <is>
-          <t>케이에스에프19호선박투자회사</t>
+          <t>코레일테크㈜</t>
         </is>
       </c>
     </row>
     <row r="514">
       <c r="A514" t="inlineStr">
         <is>
-          <t>케이에스에프1호선박투자회사</t>
+          <t>코리아메디컬홀딩스</t>
         </is>
       </c>
     </row>
     <row r="515">
       <c r="A515" t="inlineStr">
         <is>
-          <t>케이에스에프20호선박투자회사</t>
+          <t>코리아에너지터미널(주)</t>
         </is>
       </c>
     </row>
     <row r="516">
       <c r="A516" t="inlineStr">
         <is>
-          <t>케이에스에프22호선박투자회사</t>
+          <t>코미르엠지엘유한회사</t>
         </is>
       </c>
     </row>
     <row r="517">
       <c r="A517" t="inlineStr">
         <is>
-          <t>케이에스에프23호선박투자회사</t>
+          <t>코바코파트너스주식회사</t>
         </is>
       </c>
     </row>
     <row r="518">
       <c r="A518" t="inlineStr">
         <is>
-          <t>케이에스에프24호선박투자회사</t>
+          <t>코셉머티리얼㈜</t>
         </is>
       </c>
     </row>
     <row r="519">
       <c r="A519" t="inlineStr">
         <is>
-          <t>케이에스에프26호선박투자회사</t>
+          <t>코스포서비스(주)</t>
         </is>
       </c>
     </row>
     <row r="520">
       <c r="A520" t="inlineStr">
         <is>
-          <t>케이에스에프27호선박투자회사</t>
+          <t>코스포영남파워(주)</t>
         </is>
       </c>
     </row>
     <row r="521">
       <c r="A521" t="inlineStr">
         <is>
-          <t>케이에스에프28호선박투자회사</t>
+          <t>코엔바이오㈜</t>
         </is>
       </c>
     </row>
     <row r="522">
       <c r="A522" t="inlineStr">
         <is>
-          <t>케이에스에프29호선박투자회사</t>
+          <t>코웨포서비스(주)</t>
         </is>
       </c>
     </row>
     <row r="523">
       <c r="A523" t="inlineStr">
         <is>
-          <t>케이에스에프2호선박투자회사</t>
+          <t>키와파트너스㈜</t>
         </is>
       </c>
     </row>
     <row r="524">
       <c r="A524" t="inlineStr">
         <is>
-          <t>케이에스에프30호선박투자회사</t>
+          <t>탐라해상풍력발전㈜</t>
         </is>
       </c>
     </row>
     <row r="525">
       <c r="A525" t="inlineStr">
         <is>
-          <t>케이에스에프31호선박투자회사</t>
+          <t>태권도원운영관리(주)</t>
         </is>
       </c>
     </row>
     <row r="526">
       <c r="A526" t="inlineStr">
         <is>
-          <t>케이에스에프32호선박투자회사</t>
+          <t>티피에스주식회사</t>
         </is>
       </c>
     </row>
     <row r="527">
       <c r="A527" t="inlineStr">
         <is>
-          <t>케이에스에프33호선박투자회사</t>
+          <t>파주에코에너지(주)</t>
         </is>
       </c>
     </row>
     <row r="528">
       <c r="A528" t="inlineStr">
         <is>
-          <t>케이에스에프34호선박투자회사</t>
+          <t>퍼스트키퍼스㈜</t>
         </is>
       </c>
     </row>
     <row r="529">
       <c r="A529" t="inlineStr">
         <is>
-          <t>케이에스에프35호선박투자회사</t>
+          <t>피씨씨-베일리프로젝트투자조합</t>
         </is>
       </c>
     </row>
     <row r="530">
       <c r="A530" t="inlineStr">
         <is>
-          <t>케이에스에프36호선박투자회사</t>
+          <t>한강해나눔서부발전에너지전문투자형사모특별자산투자신탁(해나눔에너지펀드)</t>
         </is>
       </c>
     </row>
     <row r="531">
       <c r="A531" t="inlineStr">
         <is>
-          <t>케이에스에프37호선박투자회사</t>
+          <t>한국고벨(주)</t>
         </is>
       </c>
     </row>
     <row r="532">
       <c r="A532" t="inlineStr">
         <is>
-          <t>케이에스에프38호선박투자회사</t>
+          <t>한국공항보안주식회사</t>
         </is>
       </c>
     </row>
     <row r="533">
       <c r="A533" t="inlineStr">
         <is>
-          <t>케이에스에프39호선박투자회사</t>
+          <t>한국국제대학교행복기숙사유한회사</t>
         </is>
       </c>
     </row>
     <row r="534">
       <c r="A534" t="inlineStr">
         <is>
-          <t>케이에스에프40호선박투자회사</t>
+          <t>한국남동발전(주)</t>
         </is>
       </c>
     </row>
     <row r="535">
       <c r="A535" t="inlineStr">
         <is>
-          <t>케이에스에프41호선박투자회사</t>
+          <t>한국남부발전(주)</t>
         </is>
       </c>
     </row>
     <row r="536">
       <c r="A536" t="inlineStr">
         <is>
-          <t>케이에스에프42호선박투자회사</t>
+          <t>한국도로공사서비스</t>
         </is>
       </c>
     </row>
     <row r="537">
       <c r="A537" t="inlineStr">
         <is>
-          <t>케이에스에프43호선박투자회사</t>
+          <t>한국도로공사시설관리</t>
         </is>
       </c>
     </row>
     <row r="538">
       <c r="A538" t="inlineStr">
         <is>
-          <t>케이에스에프8호선박투자회사</t>
+          <t>한국동서발전(주)</t>
         </is>
       </c>
     </row>
     <row r="539">
       <c r="A539" t="inlineStr">
         <is>
-          <t>케이에이씨공항서비스주식회사</t>
+          <t>한국마사회시설관리(주)</t>
         </is>
       </c>
     </row>
     <row r="540">
       <c r="A540" t="inlineStr">
         <is>
-          <t>케이엔오씨서비스(주)</t>
+          <t>한국모태펀드(스포츠계정)</t>
         </is>
       </c>
     </row>
     <row r="541">
       <c r="A541" t="inlineStr">
         <is>
-          <t>케이워터기술(주)</t>
+          <t>한국문화진흥(주)</t>
         </is>
       </c>
     </row>
     <row r="542">
       <c r="A542" t="inlineStr">
         <is>
-          <t>케이워터운영관리(주)</t>
+          <t>한국벤처투자</t>
         </is>
       </c>
     </row>
     <row r="543">
       <c r="A543" t="inlineStr">
         <is>
-          <t>케이티오파트너스(주)</t>
+          <t>한국사학진흥재단행복기숙사유한회사</t>
         </is>
       </c>
     </row>
     <row r="544">
       <c r="A544" t="inlineStr">
         <is>
-          <t>케이피에스파트너스㈜</t>
+          <t>한국서부발전(주)</t>
         </is>
       </c>
     </row>
     <row r="545">
       <c r="A545" t="inlineStr">
         <is>
-          <t>케이피엑스서비스원주식회사</t>
+          <t>한국선박글로벌1호선박투자회사</t>
         </is>
       </c>
     </row>
     <row r="546">
       <c r="A546" t="inlineStr">
         <is>
-          <t>켑코솔라(주)</t>
+          <t>한국선박글로벌2호선박투자회사</t>
         </is>
       </c>
     </row>
     <row r="547">
       <c r="A547" t="inlineStr">
         <is>
-          <t>켑코이에스(주)</t>
+          <t>한국선박글로벌4호선박투자회사</t>
         </is>
       </c>
     </row>
     <row r="548">
       <c r="A548" t="inlineStr">
         <is>
-          <t>코가스보안관리(주)(주6)</t>
+          <t>한국수력원자력(주)</t>
         </is>
       </c>
     </row>
     <row r="549">
       <c r="A549" t="inlineStr">
         <is>
-          <t>코가스서비스얼라이언스(주)(주6)</t>
+          <t>한국스포츠레저(주)</t>
         </is>
       </c>
     </row>
     <row r="550">
       <c r="A550" t="inlineStr">
         <is>
-          <t>코레일관광개발㈜</t>
+          <t>한국엘엔지벙커링주식회사</t>
         </is>
       </c>
     </row>
     <row r="551">
       <c r="A551" t="inlineStr">
         <is>
-          <t>코레일네트웍스㈜</t>
+          <t>한국잡월드파트너즈(주)</t>
         </is>
       </c>
     </row>
     <row r="552">
       <c r="A552" t="inlineStr">
         <is>
-          <t>코레일로지스㈜</t>
+          <t>한국전력기술(주)</t>
         </is>
       </c>
     </row>
     <row r="553">
       <c r="A553" t="inlineStr">
         <is>
-          <t>코레일유통㈜</t>
+          <t>한국중부발전(주)</t>
         </is>
       </c>
     </row>
     <row r="554">
       <c r="A554" t="inlineStr">
         <is>
-          <t>코레일테크㈜</t>
+          <t>한국지역난방기술(주)</t>
         </is>
       </c>
     </row>
     <row r="555">
       <c r="A555" t="inlineStr">
         <is>
-          <t>코리아메디컬홀딩스</t>
+          <t>한국체육산업개발(주)</t>
         </is>
       </c>
     </row>
     <row r="556">
       <c r="A556" t="inlineStr">
         <is>
-          <t>코리아에너지터미널(주)</t>
+          <t>한국토니지102호선박투자회사</t>
         </is>
       </c>
     </row>
     <row r="557">
       <c r="A557" t="inlineStr">
         <is>
-          <t>코미르엠지엘유한회사</t>
+          <t>한국토니지103호선박투자회사</t>
         </is>
       </c>
     </row>
     <row r="558">
       <c r="A558" t="inlineStr">
         <is>
-          <t>코바코파트너스주식회사</t>
+          <t>한국토니지105호선박투자회사</t>
         </is>
       </c>
     </row>
     <row r="559">
       <c r="A559" t="inlineStr">
         <is>
-          <t>코셉머티리얼㈜</t>
+          <t>한국토니지106호선박투자회사</t>
         </is>
       </c>
     </row>
     <row r="560">
       <c r="A560" t="inlineStr">
         <is>
-          <t>코스포서비스(주)</t>
+          <t>한국토니지107호선박투자회사</t>
         </is>
       </c>
     </row>
     <row r="561">
       <c r="A561" t="inlineStr">
         <is>
-          <t>코스포영남파워(주)</t>
+          <t>한국토니지108호선박투자회사</t>
         </is>
       </c>
     </row>
     <row r="562">
       <c r="A562" t="inlineStr">
         <is>
-          <t>코엔바이오㈜</t>
+          <t>한국토니지109호선박투자회사</t>
         </is>
       </c>
     </row>
     <row r="563">
       <c r="A563" t="inlineStr">
         <is>
-          <t>코웨포서비스(주)</t>
+          <t>한국토니지110호선박투자회사</t>
         </is>
       </c>
     </row>
     <row r="564">
       <c r="A564" t="inlineStr">
         <is>
-          <t>키와파트너스㈜</t>
+          <t>한국토니지111호선박투자회사</t>
         </is>
       </c>
     </row>
     <row r="565">
       <c r="A565" t="inlineStr">
         <is>
-          <t>탐라해상풍력발전㈜</t>
+          <t>한국토니지112호선박투자회사</t>
         </is>
       </c>
     </row>
     <row r="566">
       <c r="A566" t="inlineStr">
         <is>
-          <t>태권도원운영관리(주)</t>
+          <t>한국토니지113호선박투자회사</t>
         </is>
       </c>
     </row>
     <row r="567">
       <c r="A567" t="inlineStr">
         <is>
-          <t>티피에스주식회사</t>
+          <t>한국토니지114호선박투자회사</t>
         </is>
       </c>
     </row>
     <row r="568">
       <c r="A568" t="inlineStr">
         <is>
-          <t>파주에코에너지(주)</t>
+          <t>한국토니지115호선박투자회사</t>
         </is>
       </c>
     </row>
     <row r="569">
       <c r="A569" t="inlineStr">
         <is>
-          <t>퍼스트키퍼스㈜</t>
+          <t>한국토니지116호선박투자회사</t>
         </is>
       </c>
     </row>
     <row r="570">
       <c r="A570" t="inlineStr">
         <is>
-          <t>페트라6의1호사모투자합자회사</t>
+          <t>한국토니지117호선박투자회사</t>
         </is>
       </c>
     </row>
     <row r="571">
       <c r="A571" t="inlineStr">
         <is>
-          <t>플래티넘-유망산업펀드</t>
+          <t>한국토니지118호선박투자회사</t>
         </is>
       </c>
     </row>
     <row r="572">
       <c r="A572" t="inlineStr">
         <is>
-          <t>피씨씨-베일리프로젝트투자조합</t>
+          <t>한국토니지119호선박투자회사</t>
         </is>
       </c>
     </row>
     <row r="573">
       <c r="A573" t="inlineStr">
         <is>
-          <t>하나제삼호사모투자합자회사</t>
+          <t>한국토니지120호선박투자회사</t>
         </is>
       </c>
     </row>
     <row r="574">
       <c r="A574" t="inlineStr">
         <is>
-          <t>한강해나눔서부발전에너지전문투자형사모특별자산투자신탁(해나눔에너지펀드)</t>
+          <t>한국토니지14호선박투자회사</t>
         </is>
       </c>
     </row>
     <row r="575">
       <c r="A575" t="inlineStr">
         <is>
-          <t>한국고벨(주)</t>
+          <t>한국토니지30호선박투자회사</t>
         </is>
       </c>
     </row>
     <row r="576">
       <c r="A576" t="inlineStr">
         <is>
-          <t>한국공항보안주식회사</t>
+          <t>한국토니지31호선박투자회사</t>
         </is>
       </c>
     </row>
     <row r="577">
       <c r="A577" t="inlineStr">
         <is>
-          <t>한국교육투융자회사(주)</t>
+          <t>한국토니지32호선박투자회사</t>
         </is>
       </c>
     </row>
     <row r="578">
       <c r="A578" t="inlineStr">
         <is>
-          <t>한국국제대학교행복기숙사유한회사</t>
+          <t>한국토니지33호선박투자회사</t>
         </is>
       </c>
     </row>
     <row r="579">
       <c r="A579" t="inlineStr">
         <is>
-          <t>한국남동발전(주)</t>
+          <t>한국토니지34호선박투자회사</t>
         </is>
       </c>
     </row>
     <row r="580">
       <c r="A580" t="inlineStr">
         <is>
-          <t>한국남부발전(주)</t>
+          <t>한국토니지35호선박투자회사</t>
         </is>
       </c>
     </row>
     <row r="581">
       <c r="A581" t="inlineStr">
         <is>
-          <t>한국도로공사서비스</t>
+          <t>한국토니지46호선박투자회사</t>
         </is>
       </c>
     </row>
     <row r="582">
       <c r="A582" t="inlineStr">
         <is>
-          <t>한국도로공사시설관리</t>
+          <t>한국토니지47호선박투자회사</t>
         </is>
       </c>
     </row>
     <row r="583">
       <c r="A583" t="inlineStr">
         <is>
-          <t>한국동서발전(주)</t>
+          <t>한국토니지55호선박투자회사</t>
         </is>
       </c>
     </row>
     <row r="584">
       <c r="A584" t="inlineStr">
         <is>
-          <t>한국마사회시설관리(주)</t>
+          <t>한국토니지57호선박투자회사</t>
         </is>
       </c>
     </row>
     <row r="585">
       <c r="A585" t="inlineStr">
         <is>
-          <t>한국모태펀드(스포츠계정)</t>
+          <t>한국토니지62호선박투자회사</t>
         </is>
       </c>
     </row>
     <row r="586">
       <c r="A586" t="inlineStr">
         <is>
-          <t>한국문화진흥(주)</t>
+          <t>한국토니지65호선박투자회사</t>
         </is>
       </c>
     </row>
     <row r="587">
       <c r="A587" t="inlineStr">
         <is>
-          <t>한국벤처투자</t>
+          <t>한국토니지68호선박투자회사</t>
         </is>
       </c>
     </row>
     <row r="588">
       <c r="A588" t="inlineStr">
         <is>
-          <t>한국비티엘일호투융자회사</t>
+          <t>한국토니지69호선박투자회사</t>
         </is>
       </c>
     </row>
     <row r="589">
       <c r="A589" t="inlineStr">
         <is>
-          <t>한국사학진흥재단행복기숙사유한회사</t>
+          <t>한국토니지75호선박투자회사</t>
         </is>
       </c>
     </row>
     <row r="590">
       <c r="A590" t="inlineStr">
         <is>
-          <t>한국서부발전(주)</t>
+          <t>한국토니지76호선박투자회사</t>
         </is>
       </c>
     </row>
     <row r="591">
       <c r="A591" t="inlineStr">
         <is>
-          <t>한국선박글로벌1호선박투자회사</t>
+          <t>한국토니지77호선박투자회사</t>
         </is>
       </c>
     </row>
     <row r="592">
       <c r="A592" t="inlineStr">
         <is>
-          <t>한국선박글로벌2호선박투자회사</t>
+          <t>한국토니지78호선박투자회사</t>
         </is>
       </c>
     </row>
     <row r="593">
       <c r="A593" t="inlineStr">
         <is>
-          <t>한국선박글로벌4호선박투자회사</t>
+          <t>한국토니지79호선박투자회사</t>
         </is>
       </c>
     </row>
     <row r="594">
       <c r="A594" t="inlineStr">
         <is>
-          <t>한국수력원자력(주)</t>
+          <t>한국토니지81호선박투자회사</t>
         </is>
       </c>
     </row>
     <row r="595">
       <c r="A595" t="inlineStr">
         <is>
-          <t>한국스포츠레저(주)</t>
+          <t>한국토니지82호선박투자회사</t>
         </is>
       </c>
     </row>
     <row r="596">
       <c r="A596" t="inlineStr">
         <is>
-          <t>한국엘엔지벙커링주식회사</t>
+          <t>한국토니지83호선박투자회사</t>
         </is>
       </c>
     </row>
     <row r="597">
       <c r="A597" t="inlineStr">
         <is>
-          <t>한국잡월드파트너즈(주)</t>
+          <t>한국토니지88호선박투자회사</t>
         </is>
       </c>
     </row>
     <row r="598">
       <c r="A598" t="inlineStr">
         <is>
-          <t>한국전력기술(주)</t>
+          <t>한국토니지89호선박투자회사</t>
         </is>
       </c>
     </row>
     <row r="599">
       <c r="A599" t="inlineStr">
         <is>
-          <t>한국중부발전(주)</t>
+          <t>한국토니지90호선박투자회사</t>
         </is>
       </c>
     </row>
     <row r="600">
       <c r="A600" t="inlineStr">
         <is>
-          <t>한국지역난방기술(주)</t>
+          <t>한국토니지91호선박투자회사</t>
         </is>
       </c>
     </row>
     <row r="601">
       <c r="A601" t="inlineStr">
         <is>
-          <t>한국철도일호투융자회사</t>
+          <t>한국토니지92호선박투자회사</t>
         </is>
       </c>
     </row>
     <row r="602">
       <c r="A602" t="inlineStr">
         <is>
-          <t>한국체육산업개발(주)</t>
+          <t>한국토니지93호선박투자회사</t>
         </is>
       </c>
     </row>
     <row r="603">
       <c r="A603" t="inlineStr">
         <is>
-          <t>한국토니지102호선박투자회사</t>
+          <t>한국토니지94호선박투자회사</t>
         </is>
       </c>
     </row>
     <row r="604">
       <c r="A604" t="inlineStr">
         <is>
-          <t>한국토니지103호선박투자회사</t>
+          <t>한국토니지신조10호선박투자회사</t>
         </is>
       </c>
     </row>
     <row r="605">
       <c r="A605" t="inlineStr">
         <is>
-          <t>한국토니지105호선박투자회사</t>
+          <t>한국토니지신조7호선박투자회사</t>
         </is>
       </c>
     </row>
     <row r="606">
       <c r="A606" t="inlineStr">
         <is>
-          <t>한국토니지106호선박투자회사</t>
+          <t>한국토니지신조8호선박투자회사</t>
         </is>
       </c>
     </row>
     <row r="607">
       <c r="A607" t="inlineStr">
         <is>
-          <t>한국토니지107호선박투자회사</t>
+          <t>한국토니지신조9호선박투자회사</t>
         </is>
       </c>
     </row>
     <row r="608">
       <c r="A608" t="inlineStr">
         <is>
-          <t>한국토니지108호선박투자회사</t>
+          <t>한국토지주택공사(주택도시기금)</t>
         </is>
       </c>
     </row>
     <row r="609">
       <c r="A609" t="inlineStr">
         <is>
-          <t>한국토니지109호선박투자회사</t>
+          <t>한국해상풍력(주)</t>
         </is>
       </c>
     </row>
     <row r="610">
       <c r="A610" t="inlineStr">
         <is>
-          <t>한국토니지110호선박투자회사</t>
+          <t>한국해양11호선박투자회사</t>
         </is>
       </c>
     </row>
     <row r="611">
       <c r="A611" t="inlineStr">
         <is>
-          <t>한국토니지111호선박투자회사</t>
+          <t>한국해양12호선박투자회사</t>
         </is>
       </c>
     </row>
     <row r="612">
       <c r="A612" t="inlineStr">
         <is>
-          <t>한국토니지112호선박투자회사</t>
+          <t>한국해양14호선박투자회사</t>
         </is>
       </c>
     </row>
     <row r="613">
       <c r="A613" t="inlineStr">
         <is>
-          <t>한국토니지113호선박투자회사</t>
+          <t>한국해양16호선박투자회사</t>
         </is>
       </c>
     </row>
     <row r="614">
       <c r="A614" t="inlineStr">
         <is>
-          <t>한국토니지114호선박투자회사</t>
+          <t>한국해양20호선박투자회사</t>
         </is>
       </c>
     </row>
     <row r="615">
       <c r="A615" t="inlineStr">
         <is>
-          <t>한국토니지115호선박투자회사</t>
+          <t>한국해양30호선박투자회사</t>
         </is>
       </c>
     </row>
     <row r="616">
       <c r="A616" t="inlineStr">
         <is>
-          <t>한국토니지116호선박투자회사</t>
+          <t>한국해양31호선박투자회사</t>
         </is>
       </c>
     </row>
     <row r="617">
       <c r="A617" t="inlineStr">
         <is>
-          <t>한국토니지117호선박투자회사</t>
+          <t>한국해양34호선박투자회사</t>
         </is>
       </c>
     </row>
     <row r="618">
       <c r="A618" t="inlineStr">
         <is>
-          <t>한국토니지118호선박투자회사</t>
+          <t>한국해양35호선박투자회사</t>
         </is>
       </c>
     </row>
     <row r="619">
       <c r="A619" t="inlineStr">
         <is>
-          <t>한국토니지119호선박투자회사</t>
+          <t>한국해양36호선박투자회사</t>
         </is>
       </c>
     </row>
     <row r="620">
       <c r="A620" t="inlineStr">
         <is>
-          <t>한국토니지120호선박투자회사</t>
+          <t>한국해양38호선박투자회사</t>
         </is>
       </c>
     </row>
     <row r="621">
       <c r="A621" t="inlineStr">
         <is>
-          <t>한국토니지14호선박투자회사</t>
+          <t>한국해양40호선박투자회사</t>
         </is>
       </c>
     </row>
     <row r="622">
       <c r="A622" t="inlineStr">
         <is>
-          <t>한국토니지30호선박투자회사</t>
+          <t>한국해양41호선박투자회사</t>
         </is>
       </c>
     </row>
     <row r="623">
       <c r="A623" t="inlineStr">
         <is>
-          <t>한국토니지31호선박투자회사</t>
+          <t>한국해양진흥1호선박투자회사</t>
         </is>
       </c>
     </row>
     <row r="624">
       <c r="A624" t="inlineStr">
         <is>
-          <t>한국토니지32호선박투자회사</t>
+          <t>한국해양진흥2호선박투자회사</t>
         </is>
       </c>
     </row>
     <row r="625">
       <c r="A625" t="inlineStr">
         <is>
-          <t>한국토니지33호선박투자회사</t>
+          <t>한국해양진흥3호선박투자회사</t>
         </is>
       </c>
     </row>
     <row r="626">
       <c r="A626" t="inlineStr">
         <is>
-          <t>한국토니지34호선박투자회사</t>
+          <t>한누리(주)</t>
         </is>
       </c>
     </row>
     <row r="627">
       <c r="A627" t="inlineStr">
         <is>
-          <t>한국토니지35호선박투자회사</t>
+          <t>한동대학교행복기숙사유한회사</t>
         </is>
       </c>
     </row>
     <row r="628">
       <c r="A628" t="inlineStr">
         <is>
-          <t>한국토니지46호선박투자회사</t>
+          <t>한별철강(주)</t>
         </is>
       </c>
     </row>
     <row r="629">
       <c r="A629" t="inlineStr">
         <is>
-          <t>한국토니지47호선박투자회사</t>
+          <t>한성대학교행복기숙사유한회사</t>
         </is>
       </c>
     </row>
     <row r="630">
       <c r="A630" t="inlineStr">
         <is>
-          <t>한국토니지55호선박투자회사</t>
+          <t>한양대학교행복기숙사유한회사</t>
         </is>
       </c>
     </row>
     <row r="631">
       <c r="A631" t="inlineStr">
         <is>
-          <t>한국토니지57호선박투자회사</t>
+          <t>한유원파트너스(주)</t>
         </is>
       </c>
     </row>
     <row r="632">
       <c r="A632" t="inlineStr">
         <is>
-          <t>한국토니지62호선박투자회사</t>
+          <t>한전CSC(주)</t>
         </is>
       </c>
     </row>
     <row r="633">
       <c r="A633" t="inlineStr">
         <is>
-          <t>한국토니지65호선박투자회사</t>
+          <t>한전FMS(주)</t>
         </is>
       </c>
     </row>
     <row r="634">
       <c r="A634" t="inlineStr">
         <is>
-          <t>한국토니지68호선박투자회사</t>
+          <t>한전KDN(주)</t>
         </is>
       </c>
     </row>
     <row r="635">
       <c r="A635" t="inlineStr">
         <is>
-          <t>한국토니지69호선박투자회사</t>
+          <t>한전KPS(주)</t>
         </is>
       </c>
     </row>
     <row r="636">
       <c r="A636" t="inlineStr">
         <is>
-          <t>한국토니지75호선박투자회사</t>
+          <t>한전MCS(주)</t>
         </is>
       </c>
     </row>
     <row r="637">
       <c r="A637" t="inlineStr">
         <is>
-          <t>한국토니지76호선박투자회사</t>
+          <t>한전기술서비스(주)</t>
         </is>
       </c>
     </row>
     <row r="638">
       <c r="A638" t="inlineStr">
         <is>
-          <t>한국토니지77호선박투자회사</t>
+          <t>한전원자력연료(주)</t>
         </is>
       </c>
     </row>
     <row r="639">
       <c r="A639" t="inlineStr">
         <is>
-          <t>한국토니지78호선박투자회사</t>
+          <t>합천수상태양광(주)</t>
         </is>
       </c>
     </row>
     <row r="640">
       <c r="A640" t="inlineStr">
         <is>
-          <t>한국토니지79호선박투자회사</t>
+          <t>합천수상태양광이차(주)</t>
         </is>
       </c>
     </row>
     <row r="641">
       <c r="A641" t="inlineStr">
         <is>
-          <t>한국토니지81호선박투자회사</t>
+          <t>해양신조1호선박투자회사</t>
         </is>
       </c>
     </row>
     <row r="642">
       <c r="A642" t="inlineStr">
         <is>
-          <t>한국토니지82호선박투자회사</t>
+          <t>해양신조2호선박투자회사</t>
         </is>
       </c>
     </row>
     <row r="643">
       <c r="A643" t="inlineStr">
         <is>
-          <t>한국토니지83호선박투자회사</t>
+          <t>허니팟HGI뉴투자조합</t>
         </is>
       </c>
     </row>
     <row r="644">
       <c r="A644" t="inlineStr">
         <is>
-          <t>한국토니지88호선박투자회사</t>
+          <t>헬리오스테이아벤처투자조합제1호</t>
         </is>
       </c>
     </row>
     <row r="645">
       <c r="A645" t="inlineStr">
         <is>
-          <t>한국토니지89호선박투자회사</t>
+          <t>호서대학교행복기숙사유한회사</t>
         </is>
       </c>
     </row>
     <row r="646">
       <c r="A646" t="inlineStr">
-        <is>
-          <t>한국토니지90호선박투자회사</t>
-        </is>
-      </c>
-    </row>
-    <row r="647">
-      <c r="A647" t="inlineStr">
-        <is>
-          <t>한국토니지91호선박투자회사</t>
-        </is>
-      </c>
-    </row>
-    <row r="648">
-      <c r="A648" t="inlineStr">
-        <is>
-          <t>한국토니지92호선박투자회사</t>
-        </is>
-      </c>
-    </row>
-    <row r="649">
-      <c r="A649" t="inlineStr">
-        <is>
-          <t>한국토니지93호선박투자회사</t>
-        </is>
-      </c>
-    </row>
-    <row r="650">
-      <c r="A650" t="inlineStr">
-        <is>
-          <t>한국토니지94호선박투자회사</t>
-        </is>
-      </c>
-    </row>
-    <row r="651">
-      <c r="A651" t="inlineStr">
-        <is>
-          <t>한국토니지신조10호선박투자회사</t>
-        </is>
-      </c>
-    </row>
-    <row r="652">
-      <c r="A652" t="inlineStr">
-        <is>
-          <t>한국토니지신조7호선박투자회사</t>
-        </is>
-      </c>
-    </row>
-    <row r="653">
-      <c r="A653" t="inlineStr">
-        <is>
-          <t>한국토니지신조8호선박투자회사</t>
-        </is>
-      </c>
-    </row>
-    <row r="654">
-      <c r="A654" t="inlineStr">
-        <is>
-          <t>한국토니지신조9호선박투자회사</t>
-        </is>
-      </c>
-    </row>
-    <row r="655">
-      <c r="A655" t="inlineStr">
-        <is>
-          <t>한국토지주택공사(주택도시기금)</t>
-        </is>
-      </c>
-    </row>
-    <row r="656">
-      <c r="A656" t="inlineStr">
-        <is>
-          <t>한국해상풍력(주)</t>
-        </is>
-      </c>
-    </row>
-    <row r="657">
-      <c r="A657" t="inlineStr">
-        <is>
-          <t>한국해양11호선박투자회사</t>
-        </is>
-      </c>
-    </row>
-    <row r="658">
-      <c r="A658" t="inlineStr">
-        <is>
-          <t>한국해양12호선박투자회사</t>
-        </is>
-      </c>
-    </row>
-    <row r="659">
-      <c r="A659" t="inlineStr">
-        <is>
-          <t>한국해양14호선박투자회사</t>
-        </is>
-      </c>
-    </row>
-    <row r="660">
-      <c r="A660" t="inlineStr">
-        <is>
-          <t>한국해양16호선박투자회사</t>
-        </is>
-      </c>
-    </row>
-    <row r="661">
-      <c r="A661" t="inlineStr">
-        <is>
-          <t>한국해양20호선박투자회사</t>
-        </is>
-      </c>
-    </row>
-    <row r="662">
-      <c r="A662" t="inlineStr">
-        <is>
-          <t>한국해양30호선박투자회사</t>
-        </is>
-      </c>
-    </row>
-    <row r="663">
-      <c r="A663" t="inlineStr">
-        <is>
-          <t>한국해양31호선박투자회사</t>
-        </is>
-      </c>
-    </row>
-    <row r="664">
-      <c r="A664" t="inlineStr">
-        <is>
-          <t>한국해양34호선박투자회사</t>
-        </is>
-      </c>
-    </row>
-    <row r="665">
-      <c r="A665" t="inlineStr">
-        <is>
-          <t>한국해양35호선박투자회사</t>
-        </is>
-      </c>
-    </row>
-    <row r="666">
-      <c r="A666" t="inlineStr">
-        <is>
-          <t>한국해양36호선박투자회사</t>
-        </is>
-      </c>
-    </row>
-    <row r="667">
-      <c r="A667" t="inlineStr">
-        <is>
-          <t>한국해양38호선박투자회사</t>
-        </is>
-      </c>
-    </row>
-    <row r="668">
-      <c r="A668" t="inlineStr">
-        <is>
-          <t>한국해양40호선박투자회사</t>
-        </is>
-      </c>
-    </row>
-    <row r="669">
-      <c r="A669" t="inlineStr">
-        <is>
-          <t>한국해양41호선박투자회사</t>
-        </is>
-      </c>
-    </row>
-    <row r="670">
-      <c r="A670" t="inlineStr">
-        <is>
-          <t>한국해양진흥1호선박투자회사</t>
-        </is>
-      </c>
-    </row>
-    <row r="671">
-      <c r="A671" t="inlineStr">
-        <is>
-          <t>한국해양진흥2호선박투자회사</t>
-        </is>
-      </c>
-    </row>
-    <row r="672">
-      <c r="A672" t="inlineStr">
-        <is>
-          <t>한국해양진흥3호선박투자회사</t>
-        </is>
-      </c>
-    </row>
-    <row r="673">
-      <c r="A673" t="inlineStr">
-        <is>
-          <t>한누리(주)</t>
-        </is>
-      </c>
-    </row>
-    <row r="674">
-      <c r="A674" t="inlineStr">
-        <is>
-          <t>한동대학교행복기숙사유한회사</t>
-        </is>
-      </c>
-    </row>
-    <row r="675">
-      <c r="A675" t="inlineStr">
-        <is>
-          <t>한별철강(주)</t>
-        </is>
-      </c>
-    </row>
-    <row r="676">
-      <c r="A676" t="inlineStr">
-        <is>
-          <t>한성대학교행복기숙사유한회사</t>
-        </is>
-      </c>
-    </row>
-    <row r="677">
-      <c r="A677" t="inlineStr">
-        <is>
-          <t>한양대학교행복기숙사유한회사</t>
-        </is>
-      </c>
-    </row>
-    <row r="678">
-      <c r="A678" t="inlineStr">
-        <is>
-          <t>한유원파트너스(주)</t>
-        </is>
-      </c>
-    </row>
-    <row r="679">
-      <c r="A679" t="inlineStr">
-        <is>
-          <t>한전CSC(주)</t>
-        </is>
-      </c>
-    </row>
-    <row r="680">
-      <c r="A680" t="inlineStr">
-        <is>
-          <t>한전FMS(주)</t>
-        </is>
-      </c>
-    </row>
-    <row r="681">
-      <c r="A681" t="inlineStr">
-        <is>
-          <t>한전KDN(주)</t>
-        </is>
-      </c>
-    </row>
-    <row r="682">
-      <c r="A682" t="inlineStr">
-        <is>
-          <t>한전KPS(주)</t>
-        </is>
-      </c>
-    </row>
-    <row r="683">
-      <c r="A683" t="inlineStr">
-        <is>
-          <t>한전MCS(주)</t>
-        </is>
-      </c>
-    </row>
-    <row r="684">
-      <c r="A684" t="inlineStr">
-        <is>
-          <t>한전기술서비스(주)</t>
-        </is>
-      </c>
-    </row>
-    <row r="685">
-      <c r="A685" t="inlineStr">
-        <is>
-          <t>한전원자력연료(주)</t>
-        </is>
-      </c>
-    </row>
-    <row r="686">
-      <c r="A686" t="inlineStr">
-        <is>
-          <t>합천수상태양광(주)</t>
-        </is>
-      </c>
-    </row>
-    <row r="687">
-      <c r="A687" t="inlineStr">
-        <is>
-          <t>합천수상태양광이차(주)</t>
-        </is>
-      </c>
-    </row>
-    <row r="688">
-      <c r="A688" t="inlineStr">
-        <is>
-          <t>해양신조1호선박투자회사</t>
-        </is>
-      </c>
-    </row>
-    <row r="689">
-      <c r="A689" t="inlineStr">
-        <is>
-          <t>해양신조2호선박투자회사</t>
-        </is>
-      </c>
-    </row>
-    <row r="690">
-      <c r="A690" t="inlineStr">
-        <is>
-          <t>허니팟HGI뉴투자조합</t>
-        </is>
-      </c>
-    </row>
-    <row r="691">
-      <c r="A691" t="inlineStr">
-        <is>
-          <t>헬리오스테이아벤처투자조합제1호</t>
-        </is>
-      </c>
-    </row>
-    <row r="692">
-      <c r="A692" t="inlineStr">
-        <is>
-          <t>호서대학교행복기숙사유한회사</t>
-        </is>
-      </c>
-    </row>
-    <row r="693">
-      <c r="A693" t="inlineStr">
-        <is>
-          <t>호주그린에너지제1호사모투자합자회사</t>
-        </is>
-      </c>
-    </row>
-    <row r="694">
-      <c r="A694" t="inlineStr">
         <is>
           <t>희망빛발전(주)</t>
         </is>

</xml_diff>